<commit_message>
fix(#95) Update Snomed PCE after discussion
</commit_message>
<xml_diff>
--- a/Mapping_ACRIBiSKernscoresV4.1.1.2_to_FHIR_v2027.0.0-ballot.rc1.xlsx
+++ b/Mapping_ACRIBiSKernscoresV4.1.1.2_to_FHIR_v2027.0.0-ballot.rc1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\M3nthos\Desktop\git-projects\kerndatensatz-kardiologie\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FHIRProjects\kerndatensatz-kardiologie\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCB0027C-68F3-4087-914D-ECA0D381F7B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{395CE979-4E7D-4585-86CF-F90226A7C9A5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,15 +28,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -8805,20 +8796,6 @@
 123802001 Mitral valve stenosis and regurgitation ist inaktiv, stattdessen: 194726006 Mitral stenosis with insufficiency</t>
   </si>
   <si>
-    <t xml:space="preserve">Allgemeiner Code bei Angabe von "unbehandelt" oder "unbekannt":
-73544002 "Operation on heart valve"
-Operativer Klappenersatz Code:
-34068001 "Heart valve replacement"
-Operative Klappenrekonstruktion Code:
-119769005 "Heart valve reconstruction"
-Interventionelle Klappentherapie Code:
-Postkoordiniert:
-73544002:{260507000=260519008}
----&gt;
-"Operation on heart valve:{Access=Transcatheter approach}"
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">
 300920004 "Carotid atherosclerosis"</t>
   </si>
@@ -12179,6 +12156,20 @@
 Falls nicht genauer bekannt: 
 ae &lt;=&gt; "Atherosklerotisches Ereignis" oder falls aus Item 67 bekannt, dann "eg-cv"
 aus https://simplifier.net/mii-erweiterungsmodul-kardiologie/mii-cs-kardio-atherosklerotisches-ereignis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allgemeiner Code bei Angabe von "unbehandelt" oder "unbekannt":
+73544002 "Operation on heart valve"
+Operativer Klappenersatz Code:
+34068001 "Heart valve replacement"
+Operative Klappenrekonstruktion Code:
+119769005 "Heart valve reconstruction"
+Interventionelle Klappentherapie Code:
+Postkoordiniert:
+73544002:{260507000=103388001}
+---&gt;
+"Operation on heart valve:{Access=Percutaneous approach - access}"
+</t>
   </si>
 </sst>
 </file>
@@ -13044,19 +13035,19 @@
     <xf numFmtId="0" fontId="6" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -13162,40 +13153,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -13713,6 +13670,40 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -13727,38 +13718,38 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F39296B1-D5B0-4052-943F-AEFE62BF46ED}" name="Tabelle2" displayName="Tabelle2" ref="A4:D20" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F39296B1-D5B0-4052-943F-AEFE62BF46ED}" name="Tabelle2" displayName="Tabelle2" ref="A4:D20" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
   <autoFilter ref="A4:D20" xr:uid="{F39296B1-D5B0-4052-943F-AEFE62BF46ED}"/>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{F8131921-DD04-4115-B703-859F3AE37DD0}" name="Farbcode" dataDxfId="10"/>
-    <tableColumn id="1" xr3:uid="{DEE516CC-4D04-4959-B112-344972910324}" name="Spaltenname" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{327BD4DA-EE7B-499D-A448-E17A7A314797}" name="Zweck" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{12441C76-5A10-4C2B-85B3-71C30A9C8443}" name="Beispiel" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{F8131921-DD04-4115-B703-859F3AE37DD0}" name="Farbcode" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{DEE516CC-4D04-4959-B112-344972910324}" name="Spaltenname" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{327BD4DA-EE7B-499D-A448-E17A7A314797}" name="Zweck" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{12441C76-5A10-4C2B-85B3-71C30A9C8443}" name="Beispiel" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2BCBFC2A-79C0-464A-B09B-EE9BCD198272}" name="Tabelle15" displayName="Tabelle15" ref="A1:P61" totalsRowShown="0" headerRowDxfId="33" dataDxfId="31" headerRowBorderDxfId="32" tableBorderDxfId="30" totalsRowBorderDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2BCBFC2A-79C0-464A-B09B-EE9BCD198272}" name="Tabelle15" displayName="Tabelle15" ref="A1:P61" totalsRowShown="0" headerRowDxfId="27" dataDxfId="25" headerRowBorderDxfId="26" tableBorderDxfId="24" totalsRowBorderDxfId="23">
   <autoFilter ref="A1:P61" xr:uid="{2BCBFC2A-79C0-464A-B09B-EE9BCD198272}"/>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{D5738503-B40E-4F05-BEAE-E8285BFACCAA}" name="ID" dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{77CC7209-F0DD-4FDC-970F-5FDDFC2FE5F8}" name="Parameter" dataDxfId="27"/>
-    <tableColumn id="3" xr3:uid="{9F504305-F4A9-4E65-8B38-0F0D78242D5C}" name="QuestionText" dataDxfId="26"/>
-    <tableColumn id="4" xr3:uid="{DA2B94AF-3F2B-4105-A47A-8A2AEB8C288F}" name="AnswerFormat" dataDxfId="25"/>
-    <tableColumn id="5" xr3:uid="{D4801802-F5F9-4CB1-A3F7-3138D4EBE189}" name="DataSource" dataDxfId="24"/>
-    <tableColumn id="6" xr3:uid="{8A2E9F5E-5336-4A3C-B4CB-B420B412A1EF}" name="ScoreUse" dataDxfId="23"/>
-    <tableColumn id="7" xr3:uid="{D7FED52A-0C57-4603-A125-D14E7EB786DF}" name="ParameterComment" dataDxfId="22"/>
-    <tableColumn id="8" xr3:uid="{1A96E5A2-A6E2-4B8D-969A-A997160A8941}" name="ValidValueRange" dataDxfId="21"/>
-    <tableColumn id="17" xr3:uid="{07518D5E-7FCB-43B8-95BD-7C9F5D1F9149}" name="ExampleTerminologyCodes" dataDxfId="20"/>
-    <tableColumn id="16" xr3:uid="{F30CA64E-1B7B-4843-B89D-FA7B3C94A3CA}" name="TerminologyNote" dataDxfId="19"/>
-    <tableColumn id="12" xr3:uid="{226476B6-1117-4E8F-AE46-16B8FBEBF3F1}" name="MappingRule" dataDxfId="18" dataCellStyle="Neutral"/>
-    <tableColumn id="13" xr3:uid="{1C93655F-4525-47F4-96A4-C5FCB04BC19C}" name="FHIRProfile" dataDxfId="17"/>
-    <tableColumn id="9" xr3:uid="{035B1D78-5FA8-4DEC-8B20-4784E5B12B3D}" name="FHIRElement" dataDxfId="16"/>
-    <tableColumn id="14" xr3:uid="{C95D02F6-2EE0-4575-9084-10C4A62B0378}" name="SNOMEDCode_Acribis" dataDxfId="15" dataCellStyle="Link"/>
-    <tableColumn id="10" xr3:uid="{8131AC04-20A2-41E7-8752-21B007530F96}" name="MappingNote" dataDxfId="14"/>
-    <tableColumn id="20" xr3:uid="{B278ECAC-C910-49A9-B2A3-161B1268C018}" name="ReviewAlpha3" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{D5738503-B40E-4F05-BEAE-E8285BFACCAA}" name="ID" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{77CC7209-F0DD-4FDC-970F-5FDDFC2FE5F8}" name="Parameter" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{9F504305-F4A9-4E65-8B38-0F0D78242D5C}" name="QuestionText" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{DA2B94AF-3F2B-4105-A47A-8A2AEB8C288F}" name="AnswerFormat" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{D4801802-F5F9-4CB1-A3F7-3138D4EBE189}" name="DataSource" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{8A2E9F5E-5336-4A3C-B4CB-B420B412A1EF}" name="ScoreUse" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{D7FED52A-0C57-4603-A125-D14E7EB786DF}" name="ParameterComment" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{1A96E5A2-A6E2-4B8D-969A-A997160A8941}" name="ValidValueRange" dataDxfId="15"/>
+    <tableColumn id="17" xr3:uid="{07518D5E-7FCB-43B8-95BD-7C9F5D1F9149}" name="ExampleTerminologyCodes" dataDxfId="14"/>
+    <tableColumn id="16" xr3:uid="{F30CA64E-1B7B-4843-B89D-FA7B3C94A3CA}" name="TerminologyNote" dataDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{226476B6-1117-4E8F-AE46-16B8FBEBF3F1}" name="MappingRule" dataDxfId="12" dataCellStyle="Neutral"/>
+    <tableColumn id="13" xr3:uid="{1C93655F-4525-47F4-96A4-C5FCB04BC19C}" name="FHIRProfile" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{035B1D78-5FA8-4DEC-8B20-4784E5B12B3D}" name="FHIRElement" dataDxfId="10"/>
+    <tableColumn id="14" xr3:uid="{C95D02F6-2EE0-4575-9084-10C4A62B0378}" name="SNOMEDCode_Acribis" dataDxfId="9" dataCellStyle="Link"/>
+    <tableColumn id="10" xr3:uid="{8131AC04-20A2-41E7-8752-21B007530F96}" name="MappingNote" dataDxfId="8"/>
+    <tableColumn id="20" xr3:uid="{B278ECAC-C910-49A9-B2A3-161B1268C018}" name="ReviewAlpha3" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -14073,7 +14064,7 @@
     </row>
     <row r="2" spans="1:4" ht="26.25">
       <c r="A2" s="83" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -14098,7 +14089,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="62" t="s">
-        <v>2540</v>
+        <v>2539</v>
       </c>
       <c r="D5" s="62">
         <v>5</v>
@@ -14126,7 +14117,7 @@
         <v>2</v>
       </c>
       <c r="C7" s="62" t="s">
-        <v>2542</v>
+        <v>2541</v>
       </c>
       <c r="D7" s="62" t="s">
         <v>47</v>
@@ -14140,7 +14131,7 @@
         <v>3</v>
       </c>
       <c r="C8" s="62" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="D8" s="62" t="s">
         <v>390</v>
@@ -14154,7 +14145,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="62" t="s">
-        <v>2543</v>
+        <v>2542</v>
       </c>
       <c r="D9" s="62" t="s">
         <v>49</v>
@@ -14210,7 +14201,7 @@
         <v>8</v>
       </c>
       <c r="C13" s="62" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
       <c r="D13" s="62" t="s">
         <v>52</v>
@@ -14278,7 +14269,7 @@
         <v>12</v>
       </c>
       <c r="C18" s="62" t="s">
-        <v>2471</v>
+        <v>2470</v>
       </c>
       <c r="D18" s="62" t="s">
         <v>53</v>
@@ -14306,7 +14297,7 @@
         <v>14</v>
       </c>
       <c r="C20" s="62" t="s">
-        <v>2472</v>
+        <v>2471</v>
       </c>
       <c r="D20" s="62"/>
     </row>
@@ -15199,7 +15190,7 @@
         <v>22</v>
       </c>
       <c r="L2" s="97" t="s">
-        <v>2512</v>
+        <v>2511</v>
       </c>
       <c r="M2" s="98" t="s">
         <v>23</v>
@@ -15211,10 +15202,10 @@
         <v>2426</v>
       </c>
       <c r="P2" s="56" t="s">
-        <v>2691</v>
+        <v>2690</v>
       </c>
       <c r="Q2" s="89" t="s">
-        <v>2548</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="105">
@@ -15239,10 +15230,10 @@
       </c>
       <c r="J3" s="56"/>
       <c r="K3" s="96" t="s">
-        <v>2681</v>
+        <v>2680</v>
       </c>
       <c r="L3" s="97" t="s">
-        <v>2513</v>
+        <v>2512</v>
       </c>
       <c r="M3" s="96" t="s">
         <v>28</v>
@@ -15287,7 +15278,7 @@
         <v>22</v>
       </c>
       <c r="L4" s="97" t="s">
-        <v>2512</v>
+        <v>2511</v>
       </c>
       <c r="M4" s="96" t="s">
         <v>34</v>
@@ -15334,7 +15325,7 @@
         <v>43</v>
       </c>
       <c r="L5" s="95" t="s">
-        <v>2514</v>
+        <v>2513</v>
       </c>
       <c r="M5" s="96" t="s">
         <v>44</v>
@@ -15378,19 +15369,19 @@
       </c>
       <c r="J6" s="56"/>
       <c r="K6" s="56" t="s">
-        <v>2669</v>
+        <v>2668</v>
       </c>
       <c r="L6" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M6" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N6" s="56" t="s">
         <v>53</v>
       </c>
       <c r="O6" s="55" t="s">
-        <v>2462</v>
+        <v>2461</v>
       </c>
       <c r="P6" s="100"/>
       <c r="Q6" s="68"/>
@@ -15428,10 +15419,10 @@
         <v>62</v>
       </c>
       <c r="L7" s="95" t="s">
-        <v>2507</v>
+        <v>2506</v>
       </c>
       <c r="M7" s="96" t="s">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="N7" s="96" t="s">
         <v>62</v>
@@ -15474,7 +15465,7 @@
         <v>70</v>
       </c>
       <c r="K8" s="96" t="s">
-        <v>2670</v>
+        <v>2669</v>
       </c>
       <c r="L8" s="101" t="s">
         <v>71</v>
@@ -15486,10 +15477,10 @@
         <v>73</v>
       </c>
       <c r="O8" s="55" t="s">
-        <v>2463</v>
+        <v>2462</v>
       </c>
       <c r="P8" s="56" t="s">
-        <v>2660</v>
+        <v>2659</v>
       </c>
       <c r="Q8" s="68"/>
     </row>
@@ -15525,7 +15516,7 @@
         <v>81</v>
       </c>
       <c r="K9" s="96" t="s">
-        <v>2671</v>
+        <v>2670</v>
       </c>
       <c r="L9" s="101" t="s">
         <v>83</v>
@@ -15537,10 +15528,10 @@
         <v>85</v>
       </c>
       <c r="O9" s="55" t="s">
-        <v>2464</v>
+        <v>2463</v>
       </c>
       <c r="P9" s="56" t="s">
-        <v>2659</v>
+        <v>2658</v>
       </c>
       <c r="Q9" s="2"/>
     </row>
@@ -15591,7 +15582,7 @@
         <v>93</v>
       </c>
       <c r="P10" s="56" t="s">
-        <v>2661</v>
+        <v>2660</v>
       </c>
       <c r="Q10" s="69"/>
     </row>
@@ -15625,20 +15616,20 @@
         <v>2418</v>
       </c>
       <c r="K11" s="56" t="s">
-        <v>2672</v>
+        <v>2671</v>
       </c>
       <c r="L11" s="101" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="M11" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N11" s="56" t="s">
         <v>100</v>
       </c>
       <c r="O11" s="55"/>
       <c r="P11" s="55" t="s">
-        <v>2497</v>
+        <v>2496</v>
       </c>
       <c r="Q11" s="2"/>
     </row>
@@ -15672,13 +15663,13 @@
       </c>
       <c r="J12" s="55"/>
       <c r="K12" s="55" t="s">
-        <v>2662</v>
+        <v>2661</v>
       </c>
       <c r="L12" s="95" t="s">
-        <v>2504</v>
+        <v>2503</v>
       </c>
       <c r="M12" s="102" t="s">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="N12" s="55" t="s">
         <v>107</v>
@@ -15721,13 +15712,13 @@
         <v>114</v>
       </c>
       <c r="K13" s="55" t="s">
-        <v>2665</v>
+        <v>2664</v>
       </c>
       <c r="L13" s="95" t="s">
-        <v>2504</v>
+        <v>2503</v>
       </c>
       <c r="M13" s="102" t="s">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="N13" s="102" t="s">
         <v>2454</v>
@@ -15770,22 +15761,22 @@
       </c>
       <c r="J14" s="55"/>
       <c r="K14" s="55" t="s">
-        <v>2666</v>
+        <v>2665</v>
       </c>
       <c r="L14" s="101" t="s">
-        <v>2499</v>
+        <v>2498</v>
       </c>
       <c r="M14" s="96" t="s">
         <v>121</v>
       </c>
       <c r="N14" s="96" t="s">
-        <v>2456</v>
+        <v>2696</v>
       </c>
       <c r="O14" s="55" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
       <c r="P14" s="55" t="s">
-        <v>2690</v>
+        <v>2689</v>
       </c>
       <c r="Q14" s="68"/>
     </row>
@@ -15821,13 +15812,13 @@
         <v>128</v>
       </c>
       <c r="K15" s="55" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="L15" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M15" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N15" s="58" t="s">
         <v>129</v>
@@ -15866,7 +15857,7 @@
         <v>135</v>
       </c>
       <c r="K16" s="56" t="s">
-        <v>2674</v>
+        <v>2673</v>
       </c>
       <c r="L16" s="95" t="s">
         <v>136</v>
@@ -15911,20 +15902,20 @@
         <v>144</v>
       </c>
       <c r="K17" s="56" t="s">
-        <v>2667</v>
+        <v>2666</v>
       </c>
       <c r="L17" s="95" t="s">
-        <v>2511</v>
+        <v>2510</v>
       </c>
       <c r="M17" s="56" t="s">
         <v>145</v>
       </c>
       <c r="N17" s="56" t="s">
-        <v>2500</v>
+        <v>2499</v>
       </c>
       <c r="O17" s="58"/>
       <c r="P17" s="56" t="s">
-        <v>2689</v>
+        <v>2688</v>
       </c>
       <c r="Q17" s="2"/>
     </row>
@@ -15960,22 +15951,22 @@
         <v>152</v>
       </c>
       <c r="K18" s="56" t="s">
+        <v>2674</v>
+      </c>
+      <c r="L18" s="95" t="s">
         <v>2675</v>
       </c>
-      <c r="L18" s="95" t="s">
-        <v>2676</v>
-      </c>
       <c r="M18" s="56" t="s">
-        <v>2496</v>
+        <v>2495</v>
       </c>
       <c r="N18" s="56" t="s">
-        <v>2505</v>
+        <v>2504</v>
       </c>
       <c r="O18" s="56" t="s">
         <v>153</v>
       </c>
       <c r="P18" s="56" t="s">
-        <v>2668</v>
+        <v>2667</v>
       </c>
       <c r="Q18" s="2"/>
     </row>
@@ -16011,13 +16002,13 @@
         <v>2420</v>
       </c>
       <c r="K19" s="56" t="s">
-        <v>2677</v>
+        <v>2676</v>
       </c>
       <c r="L19" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M19" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N19" s="56" t="s">
         <v>160</v>
@@ -16054,13 +16045,13 @@
       </c>
       <c r="J20" s="56"/>
       <c r="K20" s="56" t="s">
-        <v>2677</v>
+        <v>2676</v>
       </c>
       <c r="L20" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M20" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N20" s="56" t="s">
         <v>166</v>
@@ -16099,13 +16090,13 @@
         <v>2421</v>
       </c>
       <c r="K21" s="56" t="s">
-        <v>2677</v>
+        <v>2676</v>
       </c>
       <c r="L21" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M21" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N21" s="56" t="s">
         <v>172</v>
@@ -16144,16 +16135,16 @@
         <v>178</v>
       </c>
       <c r="K22" s="56" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="L22" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M22" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N22" s="102" t="s">
-        <v>2457</v>
+        <v>2456</v>
       </c>
       <c r="O22" s="56"/>
       <c r="P22" s="58"/>
@@ -16192,10 +16183,10 @@
         <v>185</v>
       </c>
       <c r="L23" s="101" t="s">
-        <v>2507</v>
+        <v>2506</v>
       </c>
       <c r="M23" s="102" t="s">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="N23" s="56" t="s">
         <v>185</v>
@@ -16236,13 +16227,13 @@
         <v>2422</v>
       </c>
       <c r="K24" s="56" t="s">
-        <v>2678</v>
+        <v>2677</v>
       </c>
       <c r="L24" s="101" t="s">
-        <v>2499</v>
+        <v>2498</v>
       </c>
       <c r="M24" s="102" t="s">
-        <v>2508</v>
+        <v>2507</v>
       </c>
       <c r="N24" s="102" t="s">
         <v>191</v>
@@ -16281,22 +16272,22 @@
       </c>
       <c r="J25" s="56"/>
       <c r="K25" s="56" t="s">
-        <v>2679</v>
+        <v>2678</v>
       </c>
       <c r="L25" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M25" s="102" t="s">
-        <v>2501</v>
+        <v>2500</v>
       </c>
       <c r="N25" s="102" t="s">
-        <v>2546</v>
+        <v>2545</v>
       </c>
       <c r="O25" s="102" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
       <c r="P25" s="102" t="s">
-        <v>2664</v>
+        <v>2663</v>
       </c>
       <c r="Q25" s="2"/>
     </row>
@@ -16333,13 +16324,13 @@
         <v>204</v>
       </c>
       <c r="L26" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M26" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N26" s="102" t="s">
-        <v>2460</v>
+        <v>2459</v>
       </c>
       <c r="O26" s="102"/>
       <c r="P26" s="58"/>
@@ -16377,7 +16368,7 @@
         <v>210</v>
       </c>
       <c r="K27" s="56" t="s">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="L27" s="95" t="s">
         <v>211</v>
@@ -16386,13 +16377,13 @@
         <v>212</v>
       </c>
       <c r="N27" s="96" t="s">
-        <v>2696</v>
+        <v>2695</v>
       </c>
       <c r="O27" s="96" t="s">
         <v>213</v>
       </c>
       <c r="P27" s="96" t="s">
-        <v>2663</v>
+        <v>2662</v>
       </c>
       <c r="Q27" s="2"/>
     </row>
@@ -16424,13 +16415,13 @@
       </c>
       <c r="J28" s="56"/>
       <c r="K28" s="56" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="L28" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M28" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N28" s="102" t="s">
         <v>219</v>
@@ -16467,13 +16458,13 @@
       </c>
       <c r="J29" s="56"/>
       <c r="K29" s="56" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="L29" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M29" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N29" s="56" t="s">
         <v>225</v>
@@ -16512,13 +16503,13 @@
         <v>231</v>
       </c>
       <c r="K30" s="56" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="L30" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M30" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N30" s="56" t="s">
         <v>232</v>
@@ -16560,10 +16551,10 @@
         <v>239</v>
       </c>
       <c r="L31" s="101" t="s">
-        <v>2507</v>
+        <v>2506</v>
       </c>
       <c r="M31" s="102" t="s">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="N31" s="102" t="s">
         <v>240</v>
@@ -16602,13 +16593,13 @@
         <v>245</v>
       </c>
       <c r="K32" s="56" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="L32" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M32" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N32" s="56" t="s">
         <v>246</v>
@@ -16645,13 +16636,13 @@
       </c>
       <c r="J33" s="56"/>
       <c r="K33" s="56" t="s">
-        <v>2677</v>
+        <v>2676</v>
       </c>
       <c r="L33" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M33" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N33" s="56" t="s">
         <v>252</v>
@@ -16690,19 +16681,19 @@
         <v>257</v>
       </c>
       <c r="K34" s="104" t="s">
-        <v>2694</v>
+        <v>2693</v>
       </c>
       <c r="L34" s="101" t="s">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="M34" s="55" t="s">
         <v>212</v>
       </c>
       <c r="N34" s="55" t="s">
-        <v>2695</v>
+        <v>2694</v>
       </c>
       <c r="O34" s="56" t="s">
-        <v>2693</v>
+        <v>2692</v>
       </c>
       <c r="P34" s="58"/>
       <c r="Q34" s="2"/>
@@ -16739,13 +16730,13 @@
         <v>263</v>
       </c>
       <c r="K35" s="56" t="s">
-        <v>2682</v>
+        <v>2681</v>
       </c>
       <c r="L35" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M35" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N35" s="56" t="s">
         <v>264</v>
@@ -16786,19 +16777,19 @@
         <v>2424</v>
       </c>
       <c r="K36" s="56" t="s">
-        <v>2683</v>
+        <v>2682</v>
       </c>
       <c r="L36" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M36" s="102" t="s">
-        <v>2509</v>
+        <v>2508</v>
       </c>
       <c r="N36" s="102" t="s">
-        <v>2461</v>
+        <v>2460</v>
       </c>
       <c r="O36" s="56" t="s">
-        <v>2467</v>
+        <v>2466</v>
       </c>
       <c r="P36" s="96"/>
       <c r="Q36" s="74"/>
@@ -16835,19 +16826,19 @@
         <v>271</v>
       </c>
       <c r="K37" s="56" t="s">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="L37" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M37" s="102" t="s">
-        <v>2509</v>
+        <v>2508</v>
       </c>
       <c r="N37" s="102" t="s">
         <v>278</v>
       </c>
       <c r="O37" s="56" t="s">
-        <v>2468</v>
+        <v>2467</v>
       </c>
       <c r="P37" s="96"/>
       <c r="Q37" s="74"/>
@@ -16884,7 +16875,7 @@
         <v>283</v>
       </c>
       <c r="K38" s="56" t="s">
-        <v>2685</v>
+        <v>2684</v>
       </c>
       <c r="L38" s="101" t="s">
         <v>284</v>
@@ -16933,22 +16924,22 @@
         <v>2425</v>
       </c>
       <c r="K39" s="56" t="s">
-        <v>2686</v>
+        <v>2685</v>
       </c>
       <c r="L39" s="101" t="s">
-        <v>2515</v>
+        <v>2514</v>
       </c>
       <c r="M39" s="102" t="s">
-        <v>2510</v>
+        <v>2509</v>
       </c>
       <c r="N39" s="114" t="s">
         <v>293</v>
       </c>
       <c r="O39" s="114" t="s">
+        <v>2686</v>
+      </c>
+      <c r="P39" s="56" t="s">
         <v>2687</v>
-      </c>
-      <c r="P39" s="56" t="s">
-        <v>2688</v>
       </c>
       <c r="Q39" s="2"/>
     </row>
@@ -16976,16 +16967,16 @@
         <v>33</v>
       </c>
       <c r="I40" s="56" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
       <c r="J40" s="56" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="K40" s="96" t="s">
         <v>298</v>
       </c>
       <c r="L40" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M40" s="102" t="s">
         <v>300</v>
@@ -16994,7 +16985,7 @@
         <v>301</v>
       </c>
       <c r="O40" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P40" s="58"/>
       <c r="Q40" s="75"/>
@@ -17030,7 +17021,7 @@
         <v>298</v>
       </c>
       <c r="L41" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M41" s="102" t="s">
         <v>300</v>
@@ -17039,7 +17030,7 @@
         <v>301</v>
       </c>
       <c r="O41" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P41" s="58"/>
       <c r="Q41" s="75"/>
@@ -17075,7 +17066,7 @@
         <v>298</v>
       </c>
       <c r="L42" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M42" s="102" t="s">
         <v>300</v>
@@ -17084,7 +17075,7 @@
         <v>301</v>
       </c>
       <c r="O42" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P42" s="58"/>
       <c r="Q42" s="2"/>
@@ -17120,7 +17111,7 @@
         <v>298</v>
       </c>
       <c r="L43" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M43" s="102" t="s">
         <v>300</v>
@@ -17129,7 +17120,7 @@
         <v>301</v>
       </c>
       <c r="O43" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P43" s="58"/>
       <c r="Q43" s="2"/>
@@ -17174,7 +17165,7 @@
         <v>301</v>
       </c>
       <c r="O44" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P44" s="58"/>
       <c r="Q44" s="2"/>
@@ -17212,7 +17203,7 @@
         <v>298</v>
       </c>
       <c r="L45" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M45" s="102" t="s">
         <v>300</v>
@@ -17221,7 +17212,7 @@
         <v>301</v>
       </c>
       <c r="O45" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P45" s="58"/>
       <c r="Q45" s="2"/>
@@ -17257,7 +17248,7 @@
         <v>298</v>
       </c>
       <c r="L46" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M46" s="102" t="s">
         <v>300</v>
@@ -17266,7 +17257,7 @@
         <v>301</v>
       </c>
       <c r="O46" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P46" s="58"/>
       <c r="Q46" s="2"/>
@@ -17302,7 +17293,7 @@
         <v>298</v>
       </c>
       <c r="L47" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M47" s="102" t="s">
         <v>300</v>
@@ -17311,7 +17302,7 @@
         <v>301</v>
       </c>
       <c r="O47" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P47" s="58"/>
       <c r="Q47" s="2"/>
@@ -17347,7 +17338,7 @@
         <v>298</v>
       </c>
       <c r="L48" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M48" s="102" t="s">
         <v>300</v>
@@ -17356,7 +17347,7 @@
         <v>301</v>
       </c>
       <c r="O48" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P48" s="58"/>
       <c r="Q48" s="2"/>
@@ -17392,7 +17383,7 @@
         <v>298</v>
       </c>
       <c r="L49" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M49" s="102" t="s">
         <v>300</v>
@@ -17401,7 +17392,7 @@
         <v>301</v>
       </c>
       <c r="O49" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P49" s="58"/>
       <c r="Q49" s="2"/>
@@ -17437,7 +17428,7 @@
         <v>298</v>
       </c>
       <c r="L50" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M50" s="102" t="s">
         <v>300</v>
@@ -17446,7 +17437,7 @@
         <v>301</v>
       </c>
       <c r="O50" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P50" s="58"/>
       <c r="Q50" s="2"/>
@@ -17482,7 +17473,7 @@
         <v>298</v>
       </c>
       <c r="L51" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M51" s="102" t="s">
         <v>300</v>
@@ -17491,7 +17482,7 @@
         <v>301</v>
       </c>
       <c r="O51" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P51" s="58"/>
       <c r="Q51" s="2"/>
@@ -17527,7 +17518,7 @@
         <v>298</v>
       </c>
       <c r="L52" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M52" s="102" t="s">
         <v>300</v>
@@ -17536,7 +17527,7 @@
         <v>301</v>
       </c>
       <c r="O52" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P52" s="58"/>
       <c r="Q52" s="2"/>
@@ -17572,7 +17563,7 @@
         <v>340</v>
       </c>
       <c r="L53" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M53" s="56" t="s">
         <v>341</v>
@@ -17617,7 +17608,7 @@
         <v>340</v>
       </c>
       <c r="L54" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M54" s="56" t="s">
         <v>341</v>
@@ -17662,7 +17653,7 @@
         <v>340</v>
       </c>
       <c r="L55" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M55" s="56" t="s">
         <v>341</v>
@@ -17707,7 +17698,7 @@
         <v>340</v>
       </c>
       <c r="L56" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M56" s="56" t="s">
         <v>341</v>
@@ -17750,7 +17741,7 @@
         <v>340</v>
       </c>
       <c r="L57" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M57" s="56" t="s">
         <v>341</v>
@@ -17759,7 +17750,7 @@
         <v>342</v>
       </c>
       <c r="O57" s="56" t="s">
-        <v>2470</v>
+        <v>2469</v>
       </c>
       <c r="P57" s="58"/>
       <c r="Q57" s="2"/>
@@ -17795,7 +17786,7 @@
         <v>340</v>
       </c>
       <c r="L58" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M58" s="56" t="s">
         <v>341</v>
@@ -17838,7 +17829,7 @@
         <v>340</v>
       </c>
       <c r="L59" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M59" s="56" t="s">
         <v>341</v>
@@ -17881,7 +17872,7 @@
         <v>340</v>
       </c>
       <c r="L60" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M60" s="56" t="s">
         <v>341</v>
@@ -17924,7 +17915,7 @@
         <v>340</v>
       </c>
       <c r="L61" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M61" s="56" t="s">
         <v>341</v>
@@ -17961,16 +17952,16 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15.75">
       <c r="A1" s="64" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
       <c r="B1" s="64" t="s">
-        <v>2570</v>
+        <v>2569</v>
       </c>
       <c r="C1" s="84" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
       <c r="D1" s="84" t="s">
-        <v>2559</v>
+        <v>2558</v>
       </c>
       <c r="E1" s="84" t="s">
         <v>386</v>
@@ -17987,13 +17978,13 @@
         <v>2452</v>
       </c>
       <c r="C2" s="86" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E2" s="86" t="s">
-        <v>2520</v>
+        <v>2519</v>
       </c>
       <c r="F2" s="85" t="s">
         <v>2444</v>
@@ -18007,13 +17998,13 @@
         <v>2429</v>
       </c>
       <c r="C3" s="86" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>2558</v>
+        <v>2557</v>
       </c>
       <c r="E3" s="85" t="s">
-        <v>2521</v>
+        <v>2520</v>
       </c>
       <c r="F3" s="85" t="s">
         <v>2445</v>
@@ -18027,31 +18018,31 @@
         <v>2429</v>
       </c>
       <c r="C4" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D4" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E4" s="86" t="s">
-        <v>2522</v>
+        <v>2521</v>
       </c>
       <c r="F4" s="86"/>
     </row>
     <row r="5" spans="1:6" ht="15.75">
       <c r="A5" s="8" t="s">
-        <v>2488</v>
+        <v>2487</v>
       </c>
       <c r="B5" s="86" t="s">
         <v>2452</v>
       </c>
       <c r="C5" s="86" t="s">
-        <v>2551</v>
+        <v>2550</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E5" s="86" t="s">
-        <v>2523</v>
+        <v>2522</v>
       </c>
       <c r="F5" s="86"/>
     </row>
@@ -18063,16 +18054,16 @@
         <v>2429</v>
       </c>
       <c r="C6" s="86" t="s">
-        <v>2556</v>
+        <v>2555</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>2567</v>
+        <v>2566</v>
       </c>
       <c r="E6" s="85" t="s">
-        <v>2524</v>
+        <v>2523</v>
       </c>
       <c r="F6" s="85" t="s">
-        <v>2560</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="126">
@@ -18083,13 +18074,13 @@
         <v>2429</v>
       </c>
       <c r="C7" s="86" t="s">
-        <v>2556</v>
+        <v>2555</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>2567</v>
+        <v>2566</v>
       </c>
       <c r="E7" s="86" t="s">
-        <v>2525</v>
+        <v>2524</v>
       </c>
       <c r="F7" s="85" t="s">
         <v>2453</v>
@@ -18103,13 +18094,13 @@
         <v>2429</v>
       </c>
       <c r="C8" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D8" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E8" t="s">
-        <v>2519</v>
+        <v>2518</v>
       </c>
       <c r="F8" s="86"/>
     </row>
@@ -18121,13 +18112,13 @@
         <v>2429</v>
       </c>
       <c r="C9" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E9" t="s">
-        <v>2491</v>
+        <v>2490</v>
       </c>
       <c r="F9" s="86"/>
     </row>
@@ -18139,16 +18130,16 @@
         <v>2429</v>
       </c>
       <c r="C10" s="86" t="s">
-        <v>2552</v>
+        <v>2551</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E10" t="s">
-        <v>2492</v>
+        <v>2491</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>2561</v>
+        <v>2560</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15.75">
@@ -18159,16 +18150,16 @@
         <v>2429</v>
       </c>
       <c r="C11" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D11" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E11" t="s">
+        <v>2492</v>
+      </c>
+      <c r="F11" t="s">
         <v>2493</v>
-      </c>
-      <c r="F11" t="s">
-        <v>2494</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="30">
@@ -18179,16 +18170,16 @@
         <v>2429</v>
       </c>
       <c r="C12" s="86" t="s">
-        <v>2551</v>
+        <v>2550</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>2558</v>
+        <v>2557</v>
       </c>
       <c r="E12" t="s">
-        <v>2535</v>
+        <v>2534</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>2562</v>
+        <v>2561</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15.75">
@@ -18199,13 +18190,13 @@
         <v>2429</v>
       </c>
       <c r="C13" s="86" t="s">
-        <v>2568</v>
+        <v>2567</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E13" t="s">
-        <v>2495</v>
+        <v>2494</v>
       </c>
       <c r="F13" s="86"/>
     </row>
@@ -18217,16 +18208,16 @@
         <v>2429</v>
       </c>
       <c r="C14" s="86" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>2569</v>
+        <v>2568</v>
       </c>
       <c r="E14" t="s">
-        <v>2534</v>
+        <v>2533</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>2563</v>
+        <v>2562</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="15.75">
@@ -18237,13 +18228,13 @@
         <v>2429</v>
       </c>
       <c r="C15" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D15" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E15" t="s">
-        <v>2533</v>
+        <v>2532</v>
       </c>
       <c r="F15" s="86"/>
     </row>
@@ -18255,16 +18246,16 @@
         <v>2429</v>
       </c>
       <c r="C16" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D16" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E16" t="s">
-        <v>2532</v>
+        <v>2531</v>
       </c>
       <c r="F16" s="85" t="s">
-        <v>2564</v>
+        <v>2563</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15.75">
@@ -18275,19 +18266,19 @@
         <v>2429</v>
       </c>
       <c r="C17" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D17" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E17" t="s">
-        <v>2531</v>
+        <v>2530</v>
       </c>
       <c r="F17" s="86"/>
     </row>
     <row r="18" spans="1:7" ht="15.75">
       <c r="A18" s="8" t="s">
-        <v>2489</v>
+        <v>2488</v>
       </c>
       <c r="B18" s="86" t="s">
         <v>2452</v>
@@ -18296,18 +18287,18 @@
         <v>2242</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E18" s="86" t="s">
-        <v>2575</v>
+        <v>2574</v>
       </c>
       <c r="F18" s="86" t="s">
-        <v>2476</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="15.75">
       <c r="A19" s="8" t="s">
-        <v>2490</v>
+        <v>2489</v>
       </c>
       <c r="B19" s="86" t="s">
         <v>2452</v>
@@ -18316,149 +18307,149 @@
         <v>2242</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E19" s="86" t="s">
-        <v>2576</v>
+        <v>2575</v>
       </c>
       <c r="F19" s="86"/>
     </row>
     <row r="20" spans="1:7" ht="47.25">
       <c r="A20" s="8" t="s">
-        <v>2487</v>
+        <v>2486</v>
       </c>
       <c r="B20" s="86" t="s">
-        <v>2473</v>
+        <v>2472</v>
       </c>
       <c r="C20" s="86" t="s">
-        <v>2556</v>
+        <v>2555</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>2571</v>
+        <v>2570</v>
       </c>
       <c r="E20" s="86" t="s">
-        <v>2577</v>
+        <v>2576</v>
       </c>
       <c r="F20" s="85" t="s">
-        <v>2565</v>
+        <v>2564</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15.75">
       <c r="A21" s="8" t="s">
-        <v>2486</v>
+        <v>2485</v>
       </c>
       <c r="B21" s="86" t="s">
-        <v>2474</v>
+        <v>2473</v>
       </c>
       <c r="C21" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D21" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E21" s="86" t="s">
-        <v>2526</v>
+        <v>2525</v>
       </c>
       <c r="F21" s="86"/>
     </row>
     <row r="22" spans="1:7" ht="15.75">
       <c r="A22" s="8" t="s">
-        <v>2483</v>
+        <v>2482</v>
       </c>
       <c r="B22" s="86" t="s">
         <v>296</v>
       </c>
       <c r="C22" s="86" t="s">
-        <v>2553</v>
+        <v>2552</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E22" s="86" t="s">
-        <v>2529</v>
+        <v>2528</v>
       </c>
       <c r="F22" s="86" t="s">
-        <v>2475</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="31.5">
       <c r="A23" s="8" t="s">
-        <v>2484</v>
+        <v>2483</v>
       </c>
       <c r="B23" s="86" t="s">
         <v>296</v>
       </c>
       <c r="C23" s="86" t="s">
-        <v>2554</v>
+        <v>2553</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E23" s="85" t="s">
-        <v>2528</v>
+        <v>2527</v>
       </c>
       <c r="F23" s="86" t="s">
-        <v>2475</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75">
       <c r="A24" s="8" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
       <c r="B24" s="86" t="s">
         <v>296</v>
       </c>
       <c r="C24" s="86" t="s">
-        <v>2555</v>
+        <v>2554</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E24" s="86" t="s">
-        <v>2527</v>
+        <v>2526</v>
       </c>
       <c r="F24" s="86" t="s">
-        <v>2475</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="15.75">
       <c r="A25" s="8" t="s">
+        <v>2478</v>
+      </c>
+      <c r="B25" s="86" t="s">
+        <v>2476</v>
+      </c>
+      <c r="C25" s="86" t="s">
+        <v>2571</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>2556</v>
+      </c>
+      <c r="E25" s="86" t="s">
+        <v>2529</v>
+      </c>
+      <c r="F25" s="86" t="s">
         <v>2479</v>
-      </c>
-      <c r="B25" s="86" t="s">
-        <v>2477</v>
-      </c>
-      <c r="C25" s="86" t="s">
-        <v>2572</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>2557</v>
-      </c>
-      <c r="E25" s="86" t="s">
-        <v>2530</v>
-      </c>
-      <c r="F25" s="86" t="s">
-        <v>2480</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="15.75">
       <c r="A26" s="8" t="s">
+        <v>2480</v>
+      </c>
+      <c r="B26" s="86" t="s">
+        <v>2477</v>
+      </c>
+      <c r="C26" s="86" t="s">
+        <v>2477</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>2572</v>
+      </c>
+      <c r="E26" s="86" t="s">
+        <v>2535</v>
+      </c>
+      <c r="F26" s="86" t="s">
         <v>2481</v>
-      </c>
-      <c r="B26" s="86" t="s">
-        <v>2478</v>
-      </c>
-      <c r="C26" s="86" t="s">
-        <v>2478</v>
-      </c>
-      <c r="D26" s="8" t="s">
-        <v>2573</v>
-      </c>
-      <c r="E26" s="86" t="s">
-        <v>2536</v>
-      </c>
-      <c r="F26" s="86" t="s">
-        <v>2482</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="47.25">
@@ -18469,14 +18460,14 @@
         <v>2429</v>
       </c>
       <c r="C27" s="86" t="s">
-        <v>2574</v>
+        <v>2573</v>
       </c>
       <c r="D27" s="86"/>
       <c r="E27" s="85" t="s">
-        <v>2537</v>
+        <v>2536</v>
       </c>
       <c r="F27" s="85" t="s">
-        <v>2566</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="15.75">
@@ -18487,11 +18478,11 @@
         <v>2451</v>
       </c>
       <c r="C28" s="86" t="s">
-        <v>2574</v>
+        <v>2573</v>
       </c>
       <c r="D28" s="86"/>
       <c r="E28" s="86" t="s">
-        <v>2538</v>
+        <v>2537</v>
       </c>
       <c r="F28" s="86"/>
     </row>
@@ -18503,11 +18494,11 @@
         <v>2451</v>
       </c>
       <c r="C29" s="86" t="s">
-        <v>2574</v>
+        <v>2573</v>
       </c>
       <c r="D29" s="86"/>
       <c r="E29" s="86" t="s">
-        <v>2539</v>
+        <v>2538</v>
       </c>
       <c r="F29" s="86"/>
     </row>
@@ -18597,19 +18588,19 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>2582</v>
+        <v>2581</v>
       </c>
       <c r="B1" t="s">
-        <v>2589</v>
+        <v>2588</v>
       </c>
       <c r="C1" t="s">
+        <v>2577</v>
+      </c>
+      <c r="D1" t="s">
         <v>2578</v>
       </c>
-      <c r="D1" t="s">
-        <v>2579</v>
-      </c>
       <c r="E1" t="s">
-        <v>2587</v>
+        <v>2586</v>
       </c>
       <c r="F1" t="s">
         <v>2327</v>
@@ -18617,532 +18608,532 @@
     </row>
     <row r="2" spans="1:6" ht="30">
       <c r="A2" s="8" t="s">
-        <v>2584</v>
+        <v>2583</v>
       </c>
       <c r="B2" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C2" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="D2" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>2652</v>
+        <v>2651</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="8" t="s">
-        <v>2583</v>
+        <v>2582</v>
       </c>
       <c r="B3" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C3" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="D3" s="91" t="s">
-        <v>2620</v>
+        <v>2619</v>
       </c>
       <c r="E3" t="s">
-        <v>2653</v>
+        <v>2652</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="8" t="s">
-        <v>2585</v>
+        <v>2584</v>
       </c>
       <c r="B4" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C4" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="D4" s="91" t="s">
-        <v>2626</v>
+        <v>2625</v>
       </c>
       <c r="E4" t="s">
-        <v>2654</v>
+        <v>2653</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="8" t="s">
-        <v>2586</v>
+        <v>2585</v>
       </c>
       <c r="B5" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C5" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="D5" s="91" t="s">
-        <v>2620</v>
+        <v>2619</v>
       </c>
       <c r="E5" t="s">
-        <v>2655</v>
+        <v>2654</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="30">
       <c r="A6" s="8" t="s">
-        <v>2588</v>
+        <v>2587</v>
       </c>
       <c r="B6" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C6" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="D6" s="91" t="s">
-        <v>2620</v>
+        <v>2619</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>2657</v>
+        <v>2656</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="8" t="s">
-        <v>2593</v>
+        <v>2592</v>
       </c>
       <c r="B7" s="90" t="s">
-        <v>2592</v>
+        <v>2591</v>
       </c>
       <c r="C7" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="D7" s="91" t="s">
-        <v>2620</v>
+        <v>2619</v>
       </c>
       <c r="E7" t="s">
-        <v>2656</v>
+        <v>2655</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="45">
       <c r="A8" s="8" t="s">
-        <v>2594</v>
+        <v>2593</v>
       </c>
       <c r="B8" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C8" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D8" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>2627</v>
+        <v>2626</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>2651</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="8" t="s">
-        <v>2595</v>
+        <v>2594</v>
       </c>
       <c r="B9" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C9" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D9" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>2628</v>
+        <v>2627</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="8" t="s">
-        <v>2596</v>
+        <v>2595</v>
       </c>
       <c r="B10" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C10" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D10" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>2629</v>
+        <v>2628</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="8" t="s">
-        <v>2597</v>
+        <v>2596</v>
       </c>
       <c r="B11" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C11" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D11" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>2630</v>
+        <v>2629</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="60">
       <c r="A12" s="8" t="s">
+        <v>2597</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2589</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2579</v>
+      </c>
+      <c r="D12" t="s">
         <v>2598</v>
       </c>
-      <c r="B12" t="s">
-        <v>2590</v>
-      </c>
-      <c r="C12" t="s">
-        <v>2580</v>
-      </c>
-      <c r="D12" t="s">
-        <v>2599</v>
-      </c>
       <c r="E12" s="10" t="s">
-        <v>2631</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="60">
       <c r="A13" s="8" t="s">
-        <v>2600</v>
+        <v>2599</v>
       </c>
       <c r="B13" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C13" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D13" t="s">
-        <v>2621</v>
+        <v>2620</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>2631</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="30">
       <c r="A14" s="8" t="s">
-        <v>2601</v>
+        <v>2600</v>
       </c>
       <c r="B14" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C14" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D14" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>2632</v>
+        <v>2631</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="8" t="s">
-        <v>2602</v>
+        <v>2601</v>
       </c>
       <c r="B15" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C15" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D15" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>2633</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="45">
       <c r="A16" s="8" t="s">
-        <v>2603</v>
+        <v>2602</v>
       </c>
       <c r="B16" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C16" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D16" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>2634</v>
+        <v>2633</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="8" t="s">
-        <v>2604</v>
+        <v>2603</v>
       </c>
       <c r="B17" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C17" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D17" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>2635</v>
+        <v>2634</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30">
       <c r="A18" s="8" t="s">
-        <v>2605</v>
+        <v>2604</v>
       </c>
       <c r="B18" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C18" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D18" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>2636</v>
+        <v>2635</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30">
       <c r="A19" s="8" t="s">
-        <v>2606</v>
+        <v>2605</v>
       </c>
       <c r="B19" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C19" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D19" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>2637</v>
+        <v>2636</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="8" t="s">
-        <v>2607</v>
+        <v>2606</v>
       </c>
       <c r="B20" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C20" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D20" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>2638</v>
+        <v>2637</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="8" t="s">
-        <v>2608</v>
+        <v>2607</v>
       </c>
       <c r="B21" s="90" t="s">
-        <v>2592</v>
+        <v>2591</v>
       </c>
       <c r="C21" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D21" s="91" t="s">
-        <v>2620</v>
+        <v>2619</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>2639</v>
+        <v>2638</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="8" t="s">
-        <v>2609</v>
+        <v>2608</v>
       </c>
       <c r="B22" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C22" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D22" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>2640</v>
+        <v>2639</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="8" t="s">
-        <v>2610</v>
+        <v>2609</v>
       </c>
       <c r="B23" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C23" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D23" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>2641</v>
+        <v>2640</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="45">
       <c r="A24" s="8" t="s">
-        <v>2611</v>
+        <v>2610</v>
       </c>
       <c r="B24" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C24" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D24" t="s">
-        <v>2622</v>
+        <v>2621</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>2642</v>
+        <v>2641</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="8" t="s">
-        <v>2612</v>
+        <v>2611</v>
       </c>
       <c r="B25" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C25" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D25" t="s">
-        <v>2622</v>
+        <v>2621</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>2643</v>
+        <v>2642</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="45">
       <c r="A26" s="8" t="s">
-        <v>2613</v>
+        <v>2612</v>
       </c>
       <c r="B26" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C26" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D26" t="s">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>2644</v>
+        <v>2643</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="8" t="s">
-        <v>2614</v>
+        <v>2613</v>
       </c>
       <c r="B27" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C27" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D27" s="91" t="s">
-        <v>2626</v>
+        <v>2625</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>2645</v>
+        <v>2644</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="30">
       <c r="A28" s="8" t="s">
-        <v>2615</v>
+        <v>2614</v>
       </c>
       <c r="B28" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C28" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D28" t="s">
-        <v>2622</v>
+        <v>2621</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>2646</v>
+        <v>2645</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="8" t="s">
-        <v>2616</v>
+        <v>2615</v>
       </c>
       <c r="B29" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C29" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D29" t="s">
-        <v>2623</v>
+        <v>2622</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>2647</v>
+        <v>2646</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="8" t="s">
-        <v>2617</v>
+        <v>2616</v>
       </c>
       <c r="B30" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C30" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D30" t="s">
-        <v>2625</v>
+        <v>2624</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>2648</v>
+        <v>2647</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="8" t="s">
-        <v>2618</v>
+        <v>2617</v>
       </c>
       <c r="B31" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C31" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D31" t="s">
-        <v>2622</v>
+        <v>2621</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>2649</v>
+        <v>2648</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="60">
       <c r="A32" s="8" t="s">
-        <v>2619</v>
+        <v>2618</v>
       </c>
       <c r="B32" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C32" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D32" t="s">
-        <v>2624</v>
+        <v>2623</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>2650</v>
+        <v>2649</v>
       </c>
     </row>
   </sheetData>
@@ -25317,10 +25308,10 @@
       <c r="E2" s="43" t="s">
         <v>1194</v>
       </c>
-      <c r="F2" s="119" t="s">
+      <c r="F2" s="120" t="s">
         <v>1195</v>
       </c>
-      <c r="G2" s="119"/>
+      <c r="G2" s="120"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="43"/>
@@ -25394,10 +25385,10 @@
       <c r="E7" s="44" t="s">
         <v>1194</v>
       </c>
-      <c r="F7" s="120" t="s">
+      <c r="F7" s="121" t="s">
         <v>1205</v>
       </c>
-      <c r="G7" s="116"/>
+      <c r="G7" s="117"/>
     </row>
     <row r="8" spans="1:7" s="44" customFormat="1">
       <c r="D8" s="44" t="s">
@@ -25406,8 +25397,8 @@
       <c r="E8" s="44" t="s">
         <v>1199</v>
       </c>
-      <c r="F8" s="120"/>
-      <c r="G8" s="116"/>
+      <c r="F8" s="121"/>
+      <c r="G8" s="117"/>
     </row>
     <row r="9" spans="1:7" s="44" customFormat="1">
       <c r="D9" s="44" t="s">
@@ -25416,8 +25407,8 @@
       <c r="E9" s="44" t="s">
         <v>1201</v>
       </c>
-      <c r="F9" s="120"/>
-      <c r="G9" s="116"/>
+      <c r="F9" s="121"/>
+      <c r="G9" s="117"/>
     </row>
     <row r="10" spans="1:7" s="44" customFormat="1">
       <c r="D10" s="44" t="s">
@@ -25426,8 +25417,8 @@
       <c r="E10" s="44" t="s">
         <v>1203</v>
       </c>
-      <c r="F10" s="120"/>
-      <c r="G10" s="116"/>
+      <c r="F10" s="121"/>
+      <c r="G10" s="117"/>
     </row>
     <row r="11" spans="1:7" s="44" customFormat="1">
       <c r="B11" s="44" t="s">
@@ -25442,8 +25433,8 @@
       <c r="E11" s="44" t="s">
         <v>1194</v>
       </c>
-      <c r="F11" s="120"/>
-      <c r="G11" s="116"/>
+      <c r="F11" s="121"/>
+      <c r="G11" s="117"/>
     </row>
     <row r="12" spans="1:7" s="44" customFormat="1">
       <c r="B12" s="44" t="s">
@@ -25452,8 +25443,8 @@
       <c r="C12" s="44" t="s">
         <v>1207</v>
       </c>
-      <c r="F12" s="120"/>
-      <c r="G12" s="116"/>
+      <c r="F12" s="121"/>
+      <c r="G12" s="117"/>
     </row>
     <row r="13" spans="1:7" s="44" customFormat="1">
       <c r="B13" s="44" t="s">
@@ -25462,8 +25453,8 @@
       <c r="C13" s="44" t="s">
         <v>1209</v>
       </c>
-      <c r="F13" s="120"/>
-      <c r="G13" s="116"/>
+      <c r="F13" s="121"/>
+      <c r="G13" s="117"/>
     </row>
     <row r="14" spans="1:7" s="43" customFormat="1">
       <c r="A14" s="43" t="s">
@@ -25475,7 +25466,7 @@
       <c r="C14" s="43" t="s">
         <v>1197</v>
       </c>
-      <c r="F14" s="121" t="s">
+      <c r="F14" s="122" t="s">
         <v>1211</v>
       </c>
       <c r="G14" s="118" t="s">
@@ -25534,10 +25525,10 @@
       </c>
       <c r="D19" s="44"/>
       <c r="E19" s="44"/>
-      <c r="F19" s="122" t="s">
+      <c r="F19" s="116" t="s">
         <v>1195</v>
       </c>
-      <c r="G19" s="116"/>
+      <c r="G19" s="117"/>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="44"/>
@@ -25549,8 +25540,8 @@
       </c>
       <c r="D20" s="44"/>
       <c r="E20" s="44"/>
-      <c r="F20" s="116"/>
-      <c r="G20" s="116"/>
+      <c r="F20" s="117"/>
+      <c r="G20" s="117"/>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="44"/>
@@ -25562,8 +25553,8 @@
       </c>
       <c r="D21" s="44"/>
       <c r="E21" s="44"/>
-      <c r="F21" s="116"/>
-      <c r="G21" s="116"/>
+      <c r="F21" s="117"/>
+      <c r="G21" s="117"/>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="44"/>
@@ -25575,8 +25566,8 @@
       </c>
       <c r="D22" s="44"/>
       <c r="E22" s="44"/>
-      <c r="F22" s="116"/>
-      <c r="G22" s="116"/>
+      <c r="F22" s="117"/>
+      <c r="G22" s="117"/>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="44"/>
@@ -25588,8 +25579,8 @@
       </c>
       <c r="D23" s="44"/>
       <c r="E23" s="44"/>
-      <c r="F23" s="116"/>
-      <c r="G23" s="116"/>
+      <c r="F23" s="117"/>
+      <c r="G23" s="117"/>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="43" t="s">
@@ -25622,10 +25613,10 @@
       </c>
       <c r="D25" s="44"/>
       <c r="E25" s="44"/>
-      <c r="F25" s="116" t="s">
+      <c r="F25" s="117" t="s">
         <v>1195</v>
       </c>
-      <c r="G25" s="123"/>
+      <c r="G25" s="119"/>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" s="44"/>
@@ -25637,8 +25628,8 @@
       </c>
       <c r="D26" s="44"/>
       <c r="E26" s="44"/>
-      <c r="F26" s="116"/>
-      <c r="G26" s="123"/>
+      <c r="F26" s="117"/>
+      <c r="G26" s="119"/>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="44"/>
@@ -25650,8 +25641,8 @@
       </c>
       <c r="D27" s="44"/>
       <c r="E27" s="44"/>
-      <c r="F27" s="116"/>
-      <c r="G27" s="123"/>
+      <c r="F27" s="117"/>
+      <c r="G27" s="119"/>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="44"/>
@@ -25663,8 +25654,8 @@
       </c>
       <c r="D28" s="44"/>
       <c r="E28" s="44"/>
-      <c r="F28" s="116"/>
-      <c r="G28" s="123"/>
+      <c r="F28" s="117"/>
+      <c r="G28" s="119"/>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" s="44"/>
@@ -25676,8 +25667,8 @@
       </c>
       <c r="D29" s="44"/>
       <c r="E29" s="44"/>
-      <c r="F29" s="116"/>
-      <c r="G29" s="123"/>
+      <c r="F29" s="117"/>
+      <c r="G29" s="119"/>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" s="44"/>
@@ -25689,8 +25680,8 @@
       </c>
       <c r="D30" s="44"/>
       <c r="E30" s="44"/>
-      <c r="F30" s="116"/>
-      <c r="G30" s="123"/>
+      <c r="F30" s="117"/>
+      <c r="G30" s="119"/>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="44"/>
@@ -25702,8 +25693,8 @@
       </c>
       <c r="D31" s="44"/>
       <c r="E31" s="44"/>
-      <c r="F31" s="116"/>
-      <c r="G31" s="123"/>
+      <c r="F31" s="117"/>
+      <c r="G31" s="119"/>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" s="43" t="s">
@@ -26141,10 +26132,10 @@
       </c>
       <c r="D64" s="44"/>
       <c r="E64" s="44"/>
-      <c r="F64" s="116" t="s">
+      <c r="F64" s="117" t="s">
         <v>1306</v>
       </c>
-      <c r="G64" s="116"/>
+      <c r="G64" s="117"/>
     </row>
     <row r="65" spans="1:7">
       <c r="A65" s="44"/>
@@ -26156,8 +26147,8 @@
       <c r="E65" s="44" t="s">
         <v>1308</v>
       </c>
-      <c r="F65" s="116"/>
-      <c r="G65" s="116"/>
+      <c r="F65" s="117"/>
+      <c r="G65" s="117"/>
     </row>
     <row r="66" spans="1:7">
       <c r="A66" s="44"/>
@@ -26169,8 +26160,8 @@
       <c r="E66" s="44" t="s">
         <v>1310</v>
       </c>
-      <c r="F66" s="116"/>
-      <c r="G66" s="116"/>
+      <c r="F66" s="117"/>
+      <c r="G66" s="117"/>
     </row>
     <row r="67" spans="1:7">
       <c r="A67" s="44"/>
@@ -26182,8 +26173,8 @@
       </c>
       <c r="D67" s="44"/>
       <c r="E67" s="44"/>
-      <c r="F67" s="116"/>
-      <c r="G67" s="116"/>
+      <c r="F67" s="117"/>
+      <c r="G67" s="117"/>
     </row>
     <row r="68" spans="1:7">
       <c r="A68" s="44"/>
@@ -26195,8 +26186,8 @@
       <c r="E68" s="44" t="s">
         <v>1314</v>
       </c>
-      <c r="F68" s="116"/>
-      <c r="G68" s="116"/>
+      <c r="F68" s="117"/>
+      <c r="G68" s="117"/>
     </row>
     <row r="69" spans="1:7">
       <c r="A69" s="44"/>
@@ -26212,8 +26203,8 @@
       <c r="E69" s="44" t="s">
         <v>1318</v>
       </c>
-      <c r="F69" s="116"/>
-      <c r="G69" s="116"/>
+      <c r="F69" s="117"/>
+      <c r="G69" s="117"/>
     </row>
     <row r="70" spans="1:7">
       <c r="A70" s="44"/>
@@ -26225,8 +26216,8 @@
       <c r="E70" s="44" t="s">
         <v>1320</v>
       </c>
-      <c r="F70" s="116"/>
-      <c r="G70" s="116"/>
+      <c r="F70" s="117"/>
+      <c r="G70" s="117"/>
     </row>
     <row r="71" spans="1:7">
       <c r="A71" s="44"/>
@@ -26238,8 +26229,8 @@
       <c r="E71" s="44" t="s">
         <v>1322</v>
       </c>
-      <c r="F71" s="116"/>
-      <c r="G71" s="116"/>
+      <c r="F71" s="117"/>
+      <c r="G71" s="117"/>
     </row>
     <row r="72" spans="1:7">
       <c r="A72" s="44"/>
@@ -26251,8 +26242,8 @@
       <c r="E72" s="44" t="s">
         <v>1324</v>
       </c>
-      <c r="F72" s="116"/>
-      <c r="G72" s="116"/>
+      <c r="F72" s="117"/>
+      <c r="G72" s="117"/>
     </row>
     <row r="73" spans="1:7">
       <c r="A73" s="44"/>
@@ -26264,8 +26255,8 @@
       <c r="E73" s="44" t="s">
         <v>1326</v>
       </c>
-      <c r="F73" s="116"/>
-      <c r="G73" s="116"/>
+      <c r="F73" s="117"/>
+      <c r="G73" s="117"/>
     </row>
     <row r="74" spans="1:7">
       <c r="A74" s="44"/>
@@ -26277,8 +26268,8 @@
       </c>
       <c r="D74" s="44"/>
       <c r="E74" s="44"/>
-      <c r="F74" s="116"/>
-      <c r="G74" s="116"/>
+      <c r="F74" s="117"/>
+      <c r="G74" s="117"/>
     </row>
     <row r="75" spans="1:7">
       <c r="A75" s="44"/>
@@ -26290,8 +26281,8 @@
       <c r="E75" s="44" t="s">
         <v>1330</v>
       </c>
-      <c r="F75" s="116"/>
-      <c r="G75" s="116"/>
+      <c r="F75" s="117"/>
+      <c r="G75" s="117"/>
     </row>
     <row r="76" spans="1:7">
       <c r="A76" s="44"/>
@@ -26307,8 +26298,8 @@
       <c r="E76" s="44" t="s">
         <v>1334</v>
       </c>
-      <c r="F76" s="116"/>
-      <c r="G76" s="116"/>
+      <c r="F76" s="117"/>
+      <c r="G76" s="117"/>
     </row>
     <row r="77" spans="1:7">
       <c r="A77" s="44"/>
@@ -26320,8 +26311,8 @@
       <c r="E77" s="44" t="s">
         <v>1336</v>
       </c>
-      <c r="F77" s="116"/>
-      <c r="G77" s="116"/>
+      <c r="F77" s="117"/>
+      <c r="G77" s="117"/>
     </row>
     <row r="78" spans="1:7">
       <c r="A78" s="44"/>
@@ -26333,8 +26324,8 @@
       <c r="E78" s="44" t="s">
         <v>1338</v>
       </c>
-      <c r="F78" s="116"/>
-      <c r="G78" s="116"/>
+      <c r="F78" s="117"/>
+      <c r="G78" s="117"/>
     </row>
     <row r="79" spans="1:7">
       <c r="A79" s="44"/>
@@ -26346,8 +26337,8 @@
       <c r="E79" s="44" t="s">
         <v>1340</v>
       </c>
-      <c r="F79" s="116"/>
-      <c r="G79" s="116"/>
+      <c r="F79" s="117"/>
+      <c r="G79" s="117"/>
     </row>
     <row r="80" spans="1:7">
       <c r="A80" s="44"/>
@@ -26359,8 +26350,8 @@
       <c r="E80" s="44" t="s">
         <v>1342</v>
       </c>
-      <c r="F80" s="116"/>
-      <c r="G80" s="116"/>
+      <c r="F80" s="117"/>
+      <c r="G80" s="117"/>
     </row>
     <row r="81" spans="1:7">
       <c r="A81" s="44"/>
@@ -26376,8 +26367,8 @@
       <c r="E81" s="44" t="s">
         <v>1346</v>
       </c>
-      <c r="F81" s="116"/>
-      <c r="G81" s="116"/>
+      <c r="F81" s="117"/>
+      <c r="G81" s="117"/>
     </row>
     <row r="82" spans="1:7">
       <c r="A82" s="44"/>
@@ -26389,8 +26380,8 @@
       <c r="E82" s="44" t="s">
         <v>1348</v>
       </c>
-      <c r="F82" s="116"/>
-      <c r="G82" s="116"/>
+      <c r="F82" s="117"/>
+      <c r="G82" s="117"/>
     </row>
     <row r="83" spans="1:7">
       <c r="A83" s="44"/>
@@ -26402,8 +26393,8 @@
       <c r="E83" s="44" t="s">
         <v>1350</v>
       </c>
-      <c r="F83" s="116"/>
-      <c r="G83" s="116"/>
+      <c r="F83" s="117"/>
+      <c r="G83" s="117"/>
     </row>
     <row r="84" spans="1:7">
       <c r="A84" s="44"/>
@@ -26415,8 +26406,8 @@
       </c>
       <c r="D84" s="44"/>
       <c r="E84" s="44"/>
-      <c r="F84" s="116"/>
-      <c r="G84" s="116"/>
+      <c r="F84" s="117"/>
+      <c r="G84" s="117"/>
     </row>
     <row r="85" spans="1:7">
       <c r="A85" s="44"/>
@@ -26428,8 +26419,8 @@
       <c r="E85" s="44" t="s">
         <v>1354</v>
       </c>
-      <c r="F85" s="116"/>
-      <c r="G85" s="116"/>
+      <c r="F85" s="117"/>
+      <c r="G85" s="117"/>
     </row>
     <row r="86" spans="1:7">
       <c r="A86" s="44"/>
@@ -26441,8 +26432,8 @@
       <c r="E86" s="44" t="s">
         <v>1356</v>
       </c>
-      <c r="F86" s="116"/>
-      <c r="G86" s="116"/>
+      <c r="F86" s="117"/>
+      <c r="G86" s="117"/>
     </row>
     <row r="87" spans="1:7">
       <c r="A87" s="44"/>
@@ -26454,8 +26445,8 @@
       <c r="E87" s="44" t="s">
         <v>1358</v>
       </c>
-      <c r="F87" s="116"/>
-      <c r="G87" s="116"/>
+      <c r="F87" s="117"/>
+      <c r="G87" s="117"/>
     </row>
     <row r="88" spans="1:7">
       <c r="A88" s="44"/>
@@ -26467,8 +26458,8 @@
       </c>
       <c r="D88" s="44"/>
       <c r="E88" s="44"/>
-      <c r="F88" s="116"/>
-      <c r="G88" s="116"/>
+      <c r="F88" s="117"/>
+      <c r="G88" s="117"/>
     </row>
     <row r="89" spans="1:7">
       <c r="A89" s="43" t="s">
@@ -26499,10 +26490,10 @@
       </c>
       <c r="D90" s="44"/>
       <c r="E90" s="44"/>
-      <c r="F90" s="116" t="s">
+      <c r="F90" s="117" t="s">
         <v>1364</v>
       </c>
-      <c r="G90" s="116"/>
+      <c r="G90" s="117"/>
     </row>
     <row r="91" spans="1:7">
       <c r="A91" s="44"/>
@@ -26514,8 +26505,8 @@
       </c>
       <c r="D91" s="44"/>
       <c r="E91" s="44"/>
-      <c r="F91" s="116"/>
-      <c r="G91" s="116"/>
+      <c r="F91" s="117"/>
+      <c r="G91" s="117"/>
     </row>
     <row r="92" spans="1:7">
       <c r="A92" s="44"/>
@@ -26527,8 +26518,8 @@
       <c r="E92" s="44" t="s">
         <v>1368</v>
       </c>
-      <c r="F92" s="116"/>
-      <c r="G92" s="116"/>
+      <c r="F92" s="117"/>
+      <c r="G92" s="117"/>
     </row>
     <row r="93" spans="1:7">
       <c r="A93" s="44"/>
@@ -26540,8 +26531,8 @@
       </c>
       <c r="D93" s="44"/>
       <c r="E93" s="44"/>
-      <c r="F93" s="116"/>
-      <c r="G93" s="116"/>
+      <c r="F93" s="117"/>
+      <c r="G93" s="117"/>
     </row>
     <row r="94" spans="1:7">
       <c r="A94" s="44"/>
@@ -26553,8 +26544,8 @@
       </c>
       <c r="D94" s="44"/>
       <c r="E94" s="44"/>
-      <c r="F94" s="116"/>
-      <c r="G94" s="116"/>
+      <c r="F94" s="117"/>
+      <c r="G94" s="117"/>
     </row>
     <row r="95" spans="1:7">
       <c r="A95" s="44"/>
@@ -26566,8 +26557,8 @@
       <c r="E95" s="44" t="s">
         <v>1374</v>
       </c>
-      <c r="F95" s="116"/>
-      <c r="G95" s="116"/>
+      <c r="F95" s="117"/>
+      <c r="G95" s="117"/>
     </row>
     <row r="96" spans="1:7">
       <c r="A96" s="44"/>
@@ -26579,8 +26570,8 @@
       <c r="E96" s="44" t="s">
         <v>1376</v>
       </c>
-      <c r="F96" s="116"/>
-      <c r="G96" s="116"/>
+      <c r="F96" s="117"/>
+      <c r="G96" s="117"/>
     </row>
     <row r="97" spans="1:7">
       <c r="A97" s="44"/>
@@ -26592,8 +26583,8 @@
       <c r="E97" s="44" t="s">
         <v>1378</v>
       </c>
-      <c r="F97" s="116"/>
-      <c r="G97" s="116"/>
+      <c r="F97" s="117"/>
+      <c r="G97" s="117"/>
     </row>
     <row r="98" spans="1:7">
       <c r="A98" s="44"/>
@@ -26605,8 +26596,8 @@
       <c r="E98" s="44" t="s">
         <v>1380</v>
       </c>
-      <c r="F98" s="116"/>
-      <c r="G98" s="116"/>
+      <c r="F98" s="117"/>
+      <c r="G98" s="117"/>
     </row>
     <row r="99" spans="1:7">
       <c r="A99" s="44"/>
@@ -26618,8 +26609,8 @@
       </c>
       <c r="D99" s="44"/>
       <c r="E99" s="44"/>
-      <c r="F99" s="116"/>
-      <c r="G99" s="116"/>
+      <c r="F99" s="117"/>
+      <c r="G99" s="117"/>
     </row>
     <row r="100" spans="1:7">
       <c r="A100" s="44"/>
@@ -26631,8 +26622,8 @@
       <c r="E100" s="44" t="s">
         <v>1384</v>
       </c>
-      <c r="F100" s="116"/>
-      <c r="G100" s="116"/>
+      <c r="F100" s="117"/>
+      <c r="G100" s="117"/>
     </row>
     <row r="101" spans="1:7">
       <c r="A101" s="44"/>
@@ -26644,8 +26635,8 @@
       <c r="E101" s="44" t="s">
         <v>1386</v>
       </c>
-      <c r="F101" s="116"/>
-      <c r="G101" s="116"/>
+      <c r="F101" s="117"/>
+      <c r="G101" s="117"/>
     </row>
     <row r="102" spans="1:7">
       <c r="A102" s="44"/>
@@ -26657,8 +26648,8 @@
       </c>
       <c r="D102" s="44"/>
       <c r="E102" s="44"/>
-      <c r="F102" s="116"/>
-      <c r="G102" s="116"/>
+      <c r="F102" s="117"/>
+      <c r="G102" s="117"/>
     </row>
     <row r="103" spans="1:7">
       <c r="A103" s="44"/>
@@ -26670,8 +26661,8 @@
       </c>
       <c r="D103" s="44"/>
       <c r="E103" s="44"/>
-      <c r="F103" s="116"/>
-      <c r="G103" s="116"/>
+      <c r="F103" s="117"/>
+      <c r="G103" s="117"/>
     </row>
     <row r="104" spans="1:7">
       <c r="A104" s="44"/>
@@ -26683,8 +26674,8 @@
       <c r="E104" s="44" t="s">
         <v>1392</v>
       </c>
-      <c r="F104" s="116"/>
-      <c r="G104" s="116"/>
+      <c r="F104" s="117"/>
+      <c r="G104" s="117"/>
     </row>
     <row r="105" spans="1:7">
       <c r="A105" s="44"/>
@@ -26696,8 +26687,8 @@
       <c r="E105" s="44" t="s">
         <v>1394</v>
       </c>
-      <c r="F105" s="116"/>
-      <c r="G105" s="116"/>
+      <c r="F105" s="117"/>
+      <c r="G105" s="117"/>
     </row>
     <row r="106" spans="1:7">
       <c r="A106" s="44"/>
@@ -26709,8 +26700,8 @@
       <c r="E106" s="44" t="s">
         <v>1199</v>
       </c>
-      <c r="F106" s="116"/>
-      <c r="G106" s="116"/>
+      <c r="F106" s="117"/>
+      <c r="G106" s="117"/>
     </row>
     <row r="107" spans="1:7">
       <c r="A107" s="44"/>
@@ -26722,8 +26713,8 @@
       <c r="E107" s="44" t="s">
         <v>1279</v>
       </c>
-      <c r="F107" s="116"/>
-      <c r="G107" s="116"/>
+      <c r="F107" s="117"/>
+      <c r="G107" s="117"/>
     </row>
     <row r="108" spans="1:7">
       <c r="A108" s="44"/>
@@ -26735,8 +26726,8 @@
       </c>
       <c r="D108" s="44"/>
       <c r="E108" s="44"/>
-      <c r="F108" s="116"/>
-      <c r="G108" s="116"/>
+      <c r="F108" s="117"/>
+      <c r="G108" s="117"/>
     </row>
     <row r="109" spans="1:7">
       <c r="A109" s="44"/>
@@ -26748,8 +26739,8 @@
       </c>
       <c r="D109" s="44"/>
       <c r="E109" s="44"/>
-      <c r="F109" s="116"/>
-      <c r="G109" s="116"/>
+      <c r="F109" s="117"/>
+      <c r="G109" s="117"/>
     </row>
     <row r="110" spans="1:7">
       <c r="A110" s="44"/>
@@ -26761,8 +26752,8 @@
       </c>
       <c r="D110" s="44"/>
       <c r="E110" s="44"/>
-      <c r="F110" s="116"/>
-      <c r="G110" s="116"/>
+      <c r="F110" s="117"/>
+      <c r="G110" s="117"/>
     </row>
     <row r="111" spans="1:7">
       <c r="A111" s="44"/>
@@ -26774,8 +26765,8 @@
       </c>
       <c r="D111" s="44"/>
       <c r="E111" s="44"/>
-      <c r="F111" s="116"/>
-      <c r="G111" s="116"/>
+      <c r="F111" s="117"/>
+      <c r="G111" s="117"/>
     </row>
     <row r="112" spans="1:7">
       <c r="A112" s="44"/>
@@ -26787,8 +26778,8 @@
       </c>
       <c r="D112" s="44"/>
       <c r="E112" s="44"/>
-      <c r="F112" s="116"/>
-      <c r="G112" s="116"/>
+      <c r="F112" s="117"/>
+      <c r="G112" s="117"/>
     </row>
     <row r="113" spans="1:7">
       <c r="A113" s="43" t="s">
@@ -26875,10 +26866,10 @@
       <c r="E118" s="44" t="s">
         <v>1419</v>
       </c>
-      <c r="F118" s="116" t="s">
+      <c r="F118" s="117" t="s">
         <v>1420</v>
       </c>
-      <c r="G118" s="116"/>
+      <c r="G118" s="117"/>
     </row>
     <row r="119" spans="1:7">
       <c r="A119" s="44"/>
@@ -26894,8 +26885,8 @@
       <c r="E119" s="44" t="s">
         <v>1424</v>
       </c>
-      <c r="F119" s="116"/>
-      <c r="G119" s="116"/>
+      <c r="F119" s="117"/>
+      <c r="G119" s="117"/>
     </row>
     <row r="120" spans="1:7">
       <c r="A120" t="s">
@@ -28380,10 +28371,10 @@
       </c>
       <c r="D279" s="44"/>
       <c r="E279" s="44"/>
-      <c r="F279" s="116" t="s">
+      <c r="F279" s="117" t="s">
         <v>1687</v>
       </c>
-      <c r="G279" s="116"/>
+      <c r="G279" s="117"/>
     </row>
     <row r="280" spans="1:7">
       <c r="A280" s="44"/>
@@ -28395,8 +28386,8 @@
       <c r="E280" s="44" t="s">
         <v>1689</v>
       </c>
-      <c r="F280" s="116"/>
-      <c r="G280" s="116"/>
+      <c r="F280" s="117"/>
+      <c r="G280" s="117"/>
     </row>
     <row r="281" spans="1:7">
       <c r="A281" s="44"/>
@@ -28408,8 +28399,8 @@
       </c>
       <c r="D281" s="44"/>
       <c r="E281" s="44"/>
-      <c r="F281" s="116"/>
-      <c r="G281" s="116"/>
+      <c r="F281" s="117"/>
+      <c r="G281" s="117"/>
     </row>
     <row r="282" spans="1:7">
       <c r="A282" s="44"/>
@@ -28425,8 +28416,8 @@
       <c r="E282" s="44" t="s">
         <v>1695</v>
       </c>
-      <c r="F282" s="116"/>
-      <c r="G282" s="116"/>
+      <c r="F282" s="117"/>
+      <c r="G282" s="117"/>
     </row>
     <row r="283" spans="1:7">
       <c r="A283" s="44"/>
@@ -28438,8 +28429,8 @@
       </c>
       <c r="D283" s="44"/>
       <c r="E283" s="44"/>
-      <c r="F283" s="116"/>
-      <c r="G283" s="116"/>
+      <c r="F283" s="117"/>
+      <c r="G283" s="117"/>
     </row>
     <row r="284" spans="1:7">
       <c r="A284" s="44"/>
@@ -28455,8 +28446,8 @@
       <c r="E284" s="44" t="s">
         <v>1701</v>
       </c>
-      <c r="F284" s="116"/>
-      <c r="G284" s="116"/>
+      <c r="F284" s="117"/>
+      <c r="G284" s="117"/>
     </row>
     <row r="285" spans="1:7">
       <c r="A285" s="44"/>
@@ -28468,8 +28459,8 @@
       <c r="E285" s="44" t="s">
         <v>1567</v>
       </c>
-      <c r="F285" s="116"/>
-      <c r="G285" s="116"/>
+      <c r="F285" s="117"/>
+      <c r="G285" s="117"/>
     </row>
     <row r="286" spans="1:7">
       <c r="A286" s="44"/>
@@ -28481,8 +28472,8 @@
       <c r="E286" s="44" t="s">
         <v>1203</v>
       </c>
-      <c r="F286" s="116"/>
-      <c r="G286" s="116"/>
+      <c r="F286" s="117"/>
+      <c r="G286" s="117"/>
     </row>
     <row r="287" spans="1:7">
       <c r="A287" s="44"/>
@@ -28494,8 +28485,8 @@
       <c r="E287" s="44" t="s">
         <v>1265</v>
       </c>
-      <c r="F287" s="116"/>
-      <c r="G287" s="116"/>
+      <c r="F287" s="117"/>
+      <c r="G287" s="117"/>
     </row>
     <row r="288" spans="1:7">
       <c r="A288" s="44"/>
@@ -28507,8 +28498,8 @@
       <c r="E288" s="44" t="s">
         <v>1281</v>
       </c>
-      <c r="F288" s="116"/>
-      <c r="G288" s="116"/>
+      <c r="F288" s="117"/>
+      <c r="G288" s="117"/>
     </row>
     <row r="289" spans="1:7">
       <c r="A289" s="44"/>
@@ -28520,8 +28511,8 @@
       <c r="E289" s="44" t="s">
         <v>1342</v>
       </c>
-      <c r="F289" s="116"/>
-      <c r="G289" s="116"/>
+      <c r="F289" s="117"/>
+      <c r="G289" s="117"/>
     </row>
     <row r="290" spans="1:7">
       <c r="A290" s="44"/>
@@ -28533,8 +28524,8 @@
       </c>
       <c r="D290" s="44"/>
       <c r="E290" s="44"/>
-      <c r="F290" s="116"/>
-      <c r="G290" s="116"/>
+      <c r="F290" s="117"/>
+      <c r="G290" s="117"/>
     </row>
     <row r="291" spans="1:7">
       <c r="A291" s="44"/>
@@ -28546,8 +28537,8 @@
       <c r="E291" s="44" t="s">
         <v>1705</v>
       </c>
-      <c r="F291" s="116"/>
-      <c r="G291" s="116"/>
+      <c r="F291" s="117"/>
+      <c r="G291" s="117"/>
     </row>
     <row r="292" spans="1:7">
       <c r="A292" s="44"/>
@@ -28559,8 +28550,8 @@
       <c r="E292" s="44" t="s">
         <v>1201</v>
       </c>
-      <c r="F292" s="116"/>
-      <c r="G292" s="116"/>
+      <c r="F292" s="117"/>
+      <c r="G292" s="117"/>
     </row>
     <row r="293" spans="1:7">
       <c r="A293" s="44"/>
@@ -28572,8 +28563,8 @@
       <c r="E293" s="44" t="s">
         <v>1571</v>
       </c>
-      <c r="F293" s="116"/>
-      <c r="G293" s="116"/>
+      <c r="F293" s="117"/>
+      <c r="G293" s="117"/>
     </row>
     <row r="294" spans="1:7">
       <c r="A294" s="44"/>
@@ -28585,8 +28576,8 @@
       <c r="E294" s="44" t="s">
         <v>1326</v>
       </c>
-      <c r="F294" s="116"/>
-      <c r="G294" s="116"/>
+      <c r="F294" s="117"/>
+      <c r="G294" s="117"/>
     </row>
     <row r="295" spans="1:7">
       <c r="A295" s="44"/>
@@ -28598,8 +28589,8 @@
       </c>
       <c r="D295" s="44"/>
       <c r="E295" s="44"/>
-      <c r="F295" s="116"/>
-      <c r="G295" s="116"/>
+      <c r="F295" s="117"/>
+      <c r="G295" s="117"/>
     </row>
     <row r="296" spans="1:7">
       <c r="A296" s="43" t="s">
@@ -28701,10 +28692,10 @@
       </c>
       <c r="D302" s="44"/>
       <c r="E302" s="44"/>
-      <c r="F302" s="116" t="s">
+      <c r="F302" s="117" t="s">
         <v>1711</v>
       </c>
-      <c r="G302" s="116" t="s">
+      <c r="G302" s="117" t="s">
         <v>1712</v>
       </c>
     </row>
@@ -28718,8 +28709,8 @@
       <c r="E303" s="44" t="s">
         <v>1689</v>
       </c>
-      <c r="F303" s="116"/>
-      <c r="G303" s="116"/>
+      <c r="F303" s="117"/>
+      <c r="G303" s="117"/>
     </row>
     <row r="304" spans="1:7">
       <c r="A304" s="43" t="s">
@@ -28925,10 +28916,10 @@
       </c>
       <c r="D316" s="44"/>
       <c r="E316" s="44"/>
-      <c r="F316" s="116" t="s">
+      <c r="F316" s="117" t="s">
         <v>1729</v>
       </c>
-      <c r="G316" s="116"/>
+      <c r="G316" s="117"/>
     </row>
     <row r="317" spans="1:7">
       <c r="A317" s="44"/>
@@ -28940,8 +28931,8 @@
       </c>
       <c r="D317" s="44"/>
       <c r="E317" s="44"/>
-      <c r="F317" s="116"/>
-      <c r="G317" s="116"/>
+      <c r="F317" s="117"/>
+      <c r="G317" s="117"/>
     </row>
     <row r="318" spans="1:7">
       <c r="A318" s="44"/>
@@ -28953,8 +28944,8 @@
       </c>
       <c r="D318" s="44"/>
       <c r="E318" s="44"/>
-      <c r="F318" s="116"/>
-      <c r="G318" s="116"/>
+      <c r="F318" s="117"/>
+      <c r="G318" s="117"/>
     </row>
     <row r="319" spans="1:7">
       <c r="A319" t="s">
@@ -30175,10 +30166,10 @@
       <c r="E450" s="44" t="s">
         <v>1981</v>
       </c>
-      <c r="F450" s="117" t="s">
+      <c r="F450" s="123" t="s">
         <v>1982</v>
       </c>
-      <c r="G450" s="116"/>
+      <c r="G450" s="117"/>
     </row>
     <row r="451" spans="1:7">
       <c r="A451" s="44"/>
@@ -30190,8 +30181,8 @@
       </c>
       <c r="D451" s="44"/>
       <c r="E451" s="44"/>
-      <c r="F451" s="117"/>
-      <c r="G451" s="116"/>
+      <c r="F451" s="123"/>
+      <c r="G451" s="117"/>
     </row>
     <row r="452" spans="1:7">
       <c r="A452" s="44"/>
@@ -30207,8 +30198,8 @@
       <c r="E452" s="44" t="s">
         <v>1988</v>
       </c>
-      <c r="F452" s="117"/>
-      <c r="G452" s="116"/>
+      <c r="F452" s="123"/>
+      <c r="G452" s="117"/>
     </row>
     <row r="453" spans="1:7">
       <c r="A453" s="44"/>
@@ -30220,8 +30211,8 @@
       <c r="E453" s="44" t="s">
         <v>1990</v>
       </c>
-      <c r="F453" s="117"/>
-      <c r="G453" s="116"/>
+      <c r="F453" s="123"/>
+      <c r="G453" s="117"/>
     </row>
     <row r="454" spans="1:7">
       <c r="A454" s="44"/>
@@ -30233,8 +30224,8 @@
       <c r="E454" s="44" t="s">
         <v>1992</v>
       </c>
-      <c r="F454" s="117"/>
-      <c r="G454" s="116"/>
+      <c r="F454" s="123"/>
+      <c r="G454" s="117"/>
     </row>
     <row r="455" spans="1:7">
       <c r="A455" s="44"/>
@@ -30246,8 +30237,8 @@
       </c>
       <c r="D455" s="44"/>
       <c r="E455" s="44"/>
-      <c r="F455" s="117"/>
-      <c r="G455" s="116"/>
+      <c r="F455" s="123"/>
+      <c r="G455" s="117"/>
     </row>
     <row r="456" spans="1:7">
       <c r="A456" s="44"/>
@@ -30259,8 +30250,8 @@
       </c>
       <c r="D456" s="44"/>
       <c r="E456" s="44"/>
-      <c r="F456" s="117"/>
-      <c r="G456" s="116"/>
+      <c r="F456" s="123"/>
+      <c r="G456" s="117"/>
     </row>
     <row r="457" spans="1:7">
       <c r="A457" s="44"/>
@@ -30272,8 +30263,8 @@
       </c>
       <c r="D457" s="44"/>
       <c r="E457" s="44"/>
-      <c r="F457" s="117"/>
-      <c r="G457" s="116"/>
+      <c r="F457" s="123"/>
+      <c r="G457" s="117"/>
     </row>
     <row r="458" spans="1:7">
       <c r="A458" s="44"/>
@@ -30285,8 +30276,8 @@
       </c>
       <c r="D458" s="44"/>
       <c r="E458" s="44"/>
-      <c r="F458" s="117"/>
-      <c r="G458" s="116"/>
+      <c r="F458" s="123"/>
+      <c r="G458" s="117"/>
     </row>
     <row r="459" spans="1:7">
       <c r="A459" s="44"/>
@@ -30298,8 +30289,8 @@
       </c>
       <c r="D459" s="44"/>
       <c r="E459" s="44"/>
-      <c r="F459" s="117"/>
-      <c r="G459" s="116"/>
+      <c r="F459" s="123"/>
+      <c r="G459" s="117"/>
     </row>
     <row r="460" spans="1:7">
       <c r="A460" s="44"/>
@@ -30311,8 +30302,8 @@
       </c>
       <c r="D460" s="44"/>
       <c r="E460" s="44"/>
-      <c r="F460" s="117"/>
-      <c r="G460" s="116"/>
+      <c r="F460" s="123"/>
+      <c r="G460" s="117"/>
     </row>
     <row r="461" spans="1:7">
       <c r="A461" s="44"/>
@@ -30324,8 +30315,8 @@
       <c r="E461" s="44" t="s">
         <v>2006</v>
       </c>
-      <c r="F461" s="117"/>
-      <c r="G461" s="116"/>
+      <c r="F461" s="123"/>
+      <c r="G461" s="117"/>
     </row>
     <row r="462" spans="1:7">
       <c r="A462" s="44"/>
@@ -30337,8 +30328,8 @@
       <c r="E462" s="44" t="s">
         <v>2008</v>
       </c>
-      <c r="F462" s="117"/>
-      <c r="G462" s="116"/>
+      <c r="F462" s="123"/>
+      <c r="G462" s="117"/>
     </row>
     <row r="463" spans="1:7">
       <c r="A463" s="44"/>
@@ -30354,8 +30345,8 @@
       <c r="E463" s="44" t="s">
         <v>2012</v>
       </c>
-      <c r="F463" s="117"/>
-      <c r="G463" s="116"/>
+      <c r="F463" s="123"/>
+      <c r="G463" s="117"/>
     </row>
     <row r="464" spans="1:7">
       <c r="A464" s="44"/>
@@ -30367,8 +30358,8 @@
       <c r="E464" s="44" t="s">
         <v>2014</v>
       </c>
-      <c r="F464" s="117"/>
-      <c r="G464" s="116"/>
+      <c r="F464" s="123"/>
+      <c r="G464" s="117"/>
     </row>
     <row r="465" spans="1:7">
       <c r="A465" s="44"/>
@@ -30380,8 +30371,8 @@
       </c>
       <c r="D465" s="44"/>
       <c r="E465" s="44"/>
-      <c r="F465" s="117"/>
-      <c r="G465" s="116"/>
+      <c r="F465" s="123"/>
+      <c r="G465" s="117"/>
     </row>
     <row r="466" spans="1:7">
       <c r="A466" s="44"/>
@@ -30393,8 +30384,8 @@
       </c>
       <c r="D466" s="44"/>
       <c r="E466" s="44"/>
-      <c r="F466" s="117"/>
-      <c r="G466" s="116"/>
+      <c r="F466" s="123"/>
+      <c r="G466" s="117"/>
     </row>
     <row r="467" spans="1:7">
       <c r="A467" s="44"/>
@@ -30406,8 +30397,8 @@
       </c>
       <c r="D467" s="44"/>
       <c r="E467" s="44"/>
-      <c r="F467" s="117"/>
-      <c r="G467" s="116"/>
+      <c r="F467" s="123"/>
+      <c r="G467" s="117"/>
     </row>
     <row r="468" spans="1:7">
       <c r="A468" s="44"/>
@@ -30419,8 +30410,8 @@
       </c>
       <c r="D468" s="44"/>
       <c r="E468" s="44"/>
-      <c r="F468" s="117"/>
-      <c r="G468" s="116"/>
+      <c r="F468" s="123"/>
+      <c r="G468" s="117"/>
     </row>
     <row r="469" spans="1:7">
       <c r="A469" s="44"/>
@@ -30432,8 +30423,8 @@
       </c>
       <c r="D469" s="44"/>
       <c r="E469" s="44"/>
-      <c r="F469" s="117"/>
-      <c r="G469" s="116"/>
+      <c r="F469" s="123"/>
+      <c r="G469" s="117"/>
     </row>
     <row r="470" spans="1:7">
       <c r="A470" s="44"/>
@@ -30445,8 +30436,8 @@
       </c>
       <c r="D470" s="44"/>
       <c r="E470" s="44"/>
-      <c r="F470" s="117"/>
-      <c r="G470" s="116"/>
+      <c r="F470" s="123"/>
+      <c r="G470" s="117"/>
     </row>
     <row r="471" spans="1:7">
       <c r="A471" s="44"/>
@@ -30458,8 +30449,8 @@
       </c>
       <c r="D471" s="44"/>
       <c r="E471" s="44"/>
-      <c r="F471" s="117"/>
-      <c r="G471" s="116"/>
+      <c r="F471" s="123"/>
+      <c r="G471" s="117"/>
     </row>
     <row r="472" spans="1:7">
       <c r="A472" s="44"/>
@@ -30471,8 +30462,8 @@
       </c>
       <c r="D472" s="44"/>
       <c r="E472" s="44"/>
-      <c r="F472" s="117"/>
-      <c r="G472" s="116"/>
+      <c r="F472" s="123"/>
+      <c r="G472" s="117"/>
     </row>
     <row r="473" spans="1:7">
       <c r="A473" s="44"/>
@@ -30484,8 +30475,8 @@
       </c>
       <c r="D473" s="44"/>
       <c r="E473" s="44"/>
-      <c r="F473" s="117"/>
-      <c r="G473" s="116"/>
+      <c r="F473" s="123"/>
+      <c r="G473" s="117"/>
     </row>
     <row r="474" spans="1:7">
       <c r="A474" s="44"/>
@@ -30501,7 +30492,7 @@
       <c r="E474" s="44" t="s">
         <v>2036</v>
       </c>
-      <c r="F474" s="117"/>
+      <c r="F474" s="123"/>
       <c r="G474" s="44"/>
     </row>
     <row r="475" spans="1:7">
@@ -30514,7 +30505,7 @@
       <c r="E475" s="44" t="s">
         <v>2038</v>
       </c>
-      <c r="F475" s="117"/>
+      <c r="F475" s="123"/>
       <c r="G475" s="44"/>
     </row>
     <row r="476" spans="1:7">
@@ -30523,7 +30514,7 @@
       <c r="C476" s="44"/>
       <c r="D476" s="44"/>
       <c r="E476" s="44"/>
-      <c r="F476" s="117"/>
+      <c r="F476" s="123"/>
       <c r="G476" s="44"/>
     </row>
     <row r="477" spans="1:7">
@@ -30695,6 +30686,22 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="F316:F318"/>
+    <mergeCell ref="G316:G318"/>
+    <mergeCell ref="F450:F476"/>
+    <mergeCell ref="G450:G473"/>
+    <mergeCell ref="F118:F119"/>
+    <mergeCell ref="G118:G119"/>
+    <mergeCell ref="F137:F139"/>
+    <mergeCell ref="G137:G139"/>
+    <mergeCell ref="F279:F295"/>
+    <mergeCell ref="G279:G295"/>
+    <mergeCell ref="F2:F6"/>
+    <mergeCell ref="G2:G6"/>
+    <mergeCell ref="F7:F13"/>
+    <mergeCell ref="G7:G13"/>
+    <mergeCell ref="F14:F18"/>
+    <mergeCell ref="G14:G18"/>
     <mergeCell ref="F19:F23"/>
     <mergeCell ref="G19:G23"/>
     <mergeCell ref="F304:F308"/>
@@ -30711,22 +30718,6 @@
     <mergeCell ref="G25:G31"/>
     <mergeCell ref="F64:F88"/>
     <mergeCell ref="G64:G88"/>
-    <mergeCell ref="F2:F6"/>
-    <mergeCell ref="G2:G6"/>
-    <mergeCell ref="F7:F13"/>
-    <mergeCell ref="G7:G13"/>
-    <mergeCell ref="F14:F18"/>
-    <mergeCell ref="G14:G18"/>
-    <mergeCell ref="F316:F318"/>
-    <mergeCell ref="G316:G318"/>
-    <mergeCell ref="F450:F476"/>
-    <mergeCell ref="G450:G473"/>
-    <mergeCell ref="F118:F119"/>
-    <mergeCell ref="G118:G119"/>
-    <mergeCell ref="F137:F139"/>
-    <mergeCell ref="G137:G139"/>
-    <mergeCell ref="F279:F295"/>
-    <mergeCell ref="G279:G295"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -31640,7 +31631,7 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
   </sheetData>
@@ -31652,6 +31643,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f" xsi:nil="true"/>
@@ -31668,16 +31668,57 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101005577104A61253744860FCC66480BADA8" ma:contentTypeVersion="18" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="63711f83cae101cfa77de3399d52e025">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="15b42a90-06dd-4669-ae82-892e5974bb2f" xmlns:ns3="c5dd6777-c59f-429e-841b-72020fd1fff4" xmlns:ns4="2d89f73c-94c0-4155-aa8d-969ee56d6579" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9da244f911df83ec31b8aa7de0186590" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="15b42a90-06dd-4669-ae82-892e5974bb2f"/>
@@ -31964,57 +32005,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8286976C-A32F-42CE-838F-E628DE116440}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E91276BE-0791-4771-952D-C50ABE3E5339}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -32032,15 +32031,15 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8286976C-A32F-42CE-838F-E628DE116440}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA3F46AF-7DEC-42CD-98A3-4934B1C64918}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9CF615A7-8B4A-4E31-8F9E-482FE203A4DA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -32058,12 +32057,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA3F46AF-7DEC-42CD-98A3-4934B1C64918}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Feature/fix katheter pce (#96)
* fix(#95) Fix SNOMED PCE for catheter operation on heart valve

* fix(#95) Update Snomed PCE after discussion
</commit_message>
<xml_diff>
--- a/Mapping_ACRIBiSKernscoresV4.1.1.2_to_FHIR_v2027.0.0-ballot.rc1.xlsx
+++ b/Mapping_ACRIBiSKernscoresV4.1.1.2_to_FHIR_v2027.0.0-ballot.rc1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\M3nthos\Desktop\git-projects\kerndatensatz-kardiologie\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FHIRProjects\kerndatensatz-kardiologie\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCB0027C-68F3-4087-914D-ECA0D381F7B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{395CE979-4E7D-4585-86CF-F90226A7C9A5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,15 +28,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -8805,20 +8796,6 @@
 123802001 Mitral valve stenosis and regurgitation ist inaktiv, stattdessen: 194726006 Mitral stenosis with insufficiency</t>
   </si>
   <si>
-    <t xml:space="preserve">Allgemeiner Code bei Angabe von "unbehandelt" oder "unbekannt":
-73544002 "Operation on heart valve"
-Operativer Klappenersatz Code:
-34068001 "Heart valve replacement"
-Operative Klappenrekonstruktion Code:
-119769005 "Heart valve reconstruction"
-Interventionelle Klappentherapie Code:
-Postkoordiniert:
-73544002:{260507000=260519008}
----&gt;
-"Operation on heart valve:{Access=Transcatheter approach}"
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">
 300920004 "Carotid atherosclerosis"</t>
   </si>
@@ -12179,6 +12156,20 @@
 Falls nicht genauer bekannt: 
 ae &lt;=&gt; "Atherosklerotisches Ereignis" oder falls aus Item 67 bekannt, dann "eg-cv"
 aus https://simplifier.net/mii-erweiterungsmodul-kardiologie/mii-cs-kardio-atherosklerotisches-ereignis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allgemeiner Code bei Angabe von "unbehandelt" oder "unbekannt":
+73544002 "Operation on heart valve"
+Operativer Klappenersatz Code:
+34068001 "Heart valve replacement"
+Operative Klappenrekonstruktion Code:
+119769005 "Heart valve reconstruction"
+Interventionelle Klappentherapie Code:
+Postkoordiniert:
+73544002:{260507000=103388001}
+---&gt;
+"Operation on heart valve:{Access=Percutaneous approach - access}"
+</t>
   </si>
 </sst>
 </file>
@@ -13044,19 +13035,19 @@
     <xf numFmtId="0" fontId="6" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -13162,40 +13153,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -13713,6 +13670,40 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -13727,38 +13718,38 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F39296B1-D5B0-4052-943F-AEFE62BF46ED}" name="Tabelle2" displayName="Tabelle2" ref="A4:D20" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F39296B1-D5B0-4052-943F-AEFE62BF46ED}" name="Tabelle2" displayName="Tabelle2" ref="A4:D20" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
   <autoFilter ref="A4:D20" xr:uid="{F39296B1-D5B0-4052-943F-AEFE62BF46ED}"/>
   <tableColumns count="4">
-    <tableColumn id="4" xr3:uid="{F8131921-DD04-4115-B703-859F3AE37DD0}" name="Farbcode" dataDxfId="10"/>
-    <tableColumn id="1" xr3:uid="{DEE516CC-4D04-4959-B112-344972910324}" name="Spaltenname" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{327BD4DA-EE7B-499D-A448-E17A7A314797}" name="Zweck" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{12441C76-5A10-4C2B-85B3-71C30A9C8443}" name="Beispiel" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{F8131921-DD04-4115-B703-859F3AE37DD0}" name="Farbcode" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{DEE516CC-4D04-4959-B112-344972910324}" name="Spaltenname" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{327BD4DA-EE7B-499D-A448-E17A7A314797}" name="Zweck" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{12441C76-5A10-4C2B-85B3-71C30A9C8443}" name="Beispiel" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2BCBFC2A-79C0-464A-B09B-EE9BCD198272}" name="Tabelle15" displayName="Tabelle15" ref="A1:P61" totalsRowShown="0" headerRowDxfId="33" dataDxfId="31" headerRowBorderDxfId="32" tableBorderDxfId="30" totalsRowBorderDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2BCBFC2A-79C0-464A-B09B-EE9BCD198272}" name="Tabelle15" displayName="Tabelle15" ref="A1:P61" totalsRowShown="0" headerRowDxfId="27" dataDxfId="25" headerRowBorderDxfId="26" tableBorderDxfId="24" totalsRowBorderDxfId="23">
   <autoFilter ref="A1:P61" xr:uid="{2BCBFC2A-79C0-464A-B09B-EE9BCD198272}"/>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{D5738503-B40E-4F05-BEAE-E8285BFACCAA}" name="ID" dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{77CC7209-F0DD-4FDC-970F-5FDDFC2FE5F8}" name="Parameter" dataDxfId="27"/>
-    <tableColumn id="3" xr3:uid="{9F504305-F4A9-4E65-8B38-0F0D78242D5C}" name="QuestionText" dataDxfId="26"/>
-    <tableColumn id="4" xr3:uid="{DA2B94AF-3F2B-4105-A47A-8A2AEB8C288F}" name="AnswerFormat" dataDxfId="25"/>
-    <tableColumn id="5" xr3:uid="{D4801802-F5F9-4CB1-A3F7-3138D4EBE189}" name="DataSource" dataDxfId="24"/>
-    <tableColumn id="6" xr3:uid="{8A2E9F5E-5336-4A3C-B4CB-B420B412A1EF}" name="ScoreUse" dataDxfId="23"/>
-    <tableColumn id="7" xr3:uid="{D7FED52A-0C57-4603-A125-D14E7EB786DF}" name="ParameterComment" dataDxfId="22"/>
-    <tableColumn id="8" xr3:uid="{1A96E5A2-A6E2-4B8D-969A-A997160A8941}" name="ValidValueRange" dataDxfId="21"/>
-    <tableColumn id="17" xr3:uid="{07518D5E-7FCB-43B8-95BD-7C9F5D1F9149}" name="ExampleTerminologyCodes" dataDxfId="20"/>
-    <tableColumn id="16" xr3:uid="{F30CA64E-1B7B-4843-B89D-FA7B3C94A3CA}" name="TerminologyNote" dataDxfId="19"/>
-    <tableColumn id="12" xr3:uid="{226476B6-1117-4E8F-AE46-16B8FBEBF3F1}" name="MappingRule" dataDxfId="18" dataCellStyle="Neutral"/>
-    <tableColumn id="13" xr3:uid="{1C93655F-4525-47F4-96A4-C5FCB04BC19C}" name="FHIRProfile" dataDxfId="17"/>
-    <tableColumn id="9" xr3:uid="{035B1D78-5FA8-4DEC-8B20-4784E5B12B3D}" name="FHIRElement" dataDxfId="16"/>
-    <tableColumn id="14" xr3:uid="{C95D02F6-2EE0-4575-9084-10C4A62B0378}" name="SNOMEDCode_Acribis" dataDxfId="15" dataCellStyle="Link"/>
-    <tableColumn id="10" xr3:uid="{8131AC04-20A2-41E7-8752-21B007530F96}" name="MappingNote" dataDxfId="14"/>
-    <tableColumn id="20" xr3:uid="{B278ECAC-C910-49A9-B2A3-161B1268C018}" name="ReviewAlpha3" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{D5738503-B40E-4F05-BEAE-E8285BFACCAA}" name="ID" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{77CC7209-F0DD-4FDC-970F-5FDDFC2FE5F8}" name="Parameter" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{9F504305-F4A9-4E65-8B38-0F0D78242D5C}" name="QuestionText" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{DA2B94AF-3F2B-4105-A47A-8A2AEB8C288F}" name="AnswerFormat" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{D4801802-F5F9-4CB1-A3F7-3138D4EBE189}" name="DataSource" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{8A2E9F5E-5336-4A3C-B4CB-B420B412A1EF}" name="ScoreUse" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{D7FED52A-0C57-4603-A125-D14E7EB786DF}" name="ParameterComment" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{1A96E5A2-A6E2-4B8D-969A-A997160A8941}" name="ValidValueRange" dataDxfId="15"/>
+    <tableColumn id="17" xr3:uid="{07518D5E-7FCB-43B8-95BD-7C9F5D1F9149}" name="ExampleTerminologyCodes" dataDxfId="14"/>
+    <tableColumn id="16" xr3:uid="{F30CA64E-1B7B-4843-B89D-FA7B3C94A3CA}" name="TerminologyNote" dataDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{226476B6-1117-4E8F-AE46-16B8FBEBF3F1}" name="MappingRule" dataDxfId="12" dataCellStyle="Neutral"/>
+    <tableColumn id="13" xr3:uid="{1C93655F-4525-47F4-96A4-C5FCB04BC19C}" name="FHIRProfile" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{035B1D78-5FA8-4DEC-8B20-4784E5B12B3D}" name="FHIRElement" dataDxfId="10"/>
+    <tableColumn id="14" xr3:uid="{C95D02F6-2EE0-4575-9084-10C4A62B0378}" name="SNOMEDCode_Acribis" dataDxfId="9" dataCellStyle="Link"/>
+    <tableColumn id="10" xr3:uid="{8131AC04-20A2-41E7-8752-21B007530F96}" name="MappingNote" dataDxfId="8"/>
+    <tableColumn id="20" xr3:uid="{B278ECAC-C910-49A9-B2A3-161B1268C018}" name="ReviewAlpha3" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -14073,7 +14064,7 @@
     </row>
     <row r="2" spans="1:4" ht="26.25">
       <c r="A2" s="83" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -14098,7 +14089,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="62" t="s">
-        <v>2540</v>
+        <v>2539</v>
       </c>
       <c r="D5" s="62">
         <v>5</v>
@@ -14126,7 +14117,7 @@
         <v>2</v>
       </c>
       <c r="C7" s="62" t="s">
-        <v>2542</v>
+        <v>2541</v>
       </c>
       <c r="D7" s="62" t="s">
         <v>47</v>
@@ -14140,7 +14131,7 @@
         <v>3</v>
       </c>
       <c r="C8" s="62" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="D8" s="62" t="s">
         <v>390</v>
@@ -14154,7 +14145,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="62" t="s">
-        <v>2543</v>
+        <v>2542</v>
       </c>
       <c r="D9" s="62" t="s">
         <v>49</v>
@@ -14210,7 +14201,7 @@
         <v>8</v>
       </c>
       <c r="C13" s="62" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
       <c r="D13" s="62" t="s">
         <v>52</v>
@@ -14278,7 +14269,7 @@
         <v>12</v>
       </c>
       <c r="C18" s="62" t="s">
-        <v>2471</v>
+        <v>2470</v>
       </c>
       <c r="D18" s="62" t="s">
         <v>53</v>
@@ -14306,7 +14297,7 @@
         <v>14</v>
       </c>
       <c r="C20" s="62" t="s">
-        <v>2472</v>
+        <v>2471</v>
       </c>
       <c r="D20" s="62"/>
     </row>
@@ -15199,7 +15190,7 @@
         <v>22</v>
       </c>
       <c r="L2" s="97" t="s">
-        <v>2512</v>
+        <v>2511</v>
       </c>
       <c r="M2" s="98" t="s">
         <v>23</v>
@@ -15211,10 +15202,10 @@
         <v>2426</v>
       </c>
       <c r="P2" s="56" t="s">
-        <v>2691</v>
+        <v>2690</v>
       </c>
       <c r="Q2" s="89" t="s">
-        <v>2548</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="105">
@@ -15239,10 +15230,10 @@
       </c>
       <c r="J3" s="56"/>
       <c r="K3" s="96" t="s">
-        <v>2681</v>
+        <v>2680</v>
       </c>
       <c r="L3" s="97" t="s">
-        <v>2513</v>
+        <v>2512</v>
       </c>
       <c r="M3" s="96" t="s">
         <v>28</v>
@@ -15287,7 +15278,7 @@
         <v>22</v>
       </c>
       <c r="L4" s="97" t="s">
-        <v>2512</v>
+        <v>2511</v>
       </c>
       <c r="M4" s="96" t="s">
         <v>34</v>
@@ -15334,7 +15325,7 @@
         <v>43</v>
       </c>
       <c r="L5" s="95" t="s">
-        <v>2514</v>
+        <v>2513</v>
       </c>
       <c r="M5" s="96" t="s">
         <v>44</v>
@@ -15378,19 +15369,19 @@
       </c>
       <c r="J6" s="56"/>
       <c r="K6" s="56" t="s">
-        <v>2669</v>
+        <v>2668</v>
       </c>
       <c r="L6" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M6" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N6" s="56" t="s">
         <v>53</v>
       </c>
       <c r="O6" s="55" t="s">
-        <v>2462</v>
+        <v>2461</v>
       </c>
       <c r="P6" s="100"/>
       <c r="Q6" s="68"/>
@@ -15428,10 +15419,10 @@
         <v>62</v>
       </c>
       <c r="L7" s="95" t="s">
-        <v>2507</v>
+        <v>2506</v>
       </c>
       <c r="M7" s="96" t="s">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="N7" s="96" t="s">
         <v>62</v>
@@ -15474,7 +15465,7 @@
         <v>70</v>
       </c>
       <c r="K8" s="96" t="s">
-        <v>2670</v>
+        <v>2669</v>
       </c>
       <c r="L8" s="101" t="s">
         <v>71</v>
@@ -15486,10 +15477,10 @@
         <v>73</v>
       </c>
       <c r="O8" s="55" t="s">
-        <v>2463</v>
+        <v>2462</v>
       </c>
       <c r="P8" s="56" t="s">
-        <v>2660</v>
+        <v>2659</v>
       </c>
       <c r="Q8" s="68"/>
     </row>
@@ -15525,7 +15516,7 @@
         <v>81</v>
       </c>
       <c r="K9" s="96" t="s">
-        <v>2671</v>
+        <v>2670</v>
       </c>
       <c r="L9" s="101" t="s">
         <v>83</v>
@@ -15537,10 +15528,10 @@
         <v>85</v>
       </c>
       <c r="O9" s="55" t="s">
-        <v>2464</v>
+        <v>2463</v>
       </c>
       <c r="P9" s="56" t="s">
-        <v>2659</v>
+        <v>2658</v>
       </c>
       <c r="Q9" s="2"/>
     </row>
@@ -15591,7 +15582,7 @@
         <v>93</v>
       </c>
       <c r="P10" s="56" t="s">
-        <v>2661</v>
+        <v>2660</v>
       </c>
       <c r="Q10" s="69"/>
     </row>
@@ -15625,20 +15616,20 @@
         <v>2418</v>
       </c>
       <c r="K11" s="56" t="s">
-        <v>2672</v>
+        <v>2671</v>
       </c>
       <c r="L11" s="101" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="M11" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N11" s="56" t="s">
         <v>100</v>
       </c>
       <c r="O11" s="55"/>
       <c r="P11" s="55" t="s">
-        <v>2497</v>
+        <v>2496</v>
       </c>
       <c r="Q11" s="2"/>
     </row>
@@ -15672,13 +15663,13 @@
       </c>
       <c r="J12" s="55"/>
       <c r="K12" s="55" t="s">
-        <v>2662</v>
+        <v>2661</v>
       </c>
       <c r="L12" s="95" t="s">
-        <v>2504</v>
+        <v>2503</v>
       </c>
       <c r="M12" s="102" t="s">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="N12" s="55" t="s">
         <v>107</v>
@@ -15721,13 +15712,13 @@
         <v>114</v>
       </c>
       <c r="K13" s="55" t="s">
-        <v>2665</v>
+        <v>2664</v>
       </c>
       <c r="L13" s="95" t="s">
-        <v>2504</v>
+        <v>2503</v>
       </c>
       <c r="M13" s="102" t="s">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="N13" s="102" t="s">
         <v>2454</v>
@@ -15770,22 +15761,22 @@
       </c>
       <c r="J14" s="55"/>
       <c r="K14" s="55" t="s">
-        <v>2666</v>
+        <v>2665</v>
       </c>
       <c r="L14" s="101" t="s">
-        <v>2499</v>
+        <v>2498</v>
       </c>
       <c r="M14" s="96" t="s">
         <v>121</v>
       </c>
       <c r="N14" s="96" t="s">
-        <v>2456</v>
+        <v>2696</v>
       </c>
       <c r="O14" s="55" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
       <c r="P14" s="55" t="s">
-        <v>2690</v>
+        <v>2689</v>
       </c>
       <c r="Q14" s="68"/>
     </row>
@@ -15821,13 +15812,13 @@
         <v>128</v>
       </c>
       <c r="K15" s="55" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="L15" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M15" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N15" s="58" t="s">
         <v>129</v>
@@ -15866,7 +15857,7 @@
         <v>135</v>
       </c>
       <c r="K16" s="56" t="s">
-        <v>2674</v>
+        <v>2673</v>
       </c>
       <c r="L16" s="95" t="s">
         <v>136</v>
@@ -15911,20 +15902,20 @@
         <v>144</v>
       </c>
       <c r="K17" s="56" t="s">
-        <v>2667</v>
+        <v>2666</v>
       </c>
       <c r="L17" s="95" t="s">
-        <v>2511</v>
+        <v>2510</v>
       </c>
       <c r="M17" s="56" t="s">
         <v>145</v>
       </c>
       <c r="N17" s="56" t="s">
-        <v>2500</v>
+        <v>2499</v>
       </c>
       <c r="O17" s="58"/>
       <c r="P17" s="56" t="s">
-        <v>2689</v>
+        <v>2688</v>
       </c>
       <c r="Q17" s="2"/>
     </row>
@@ -15960,22 +15951,22 @@
         <v>152</v>
       </c>
       <c r="K18" s="56" t="s">
+        <v>2674</v>
+      </c>
+      <c r="L18" s="95" t="s">
         <v>2675</v>
       </c>
-      <c r="L18" s="95" t="s">
-        <v>2676</v>
-      </c>
       <c r="M18" s="56" t="s">
-        <v>2496</v>
+        <v>2495</v>
       </c>
       <c r="N18" s="56" t="s">
-        <v>2505</v>
+        <v>2504</v>
       </c>
       <c r="O18" s="56" t="s">
         <v>153</v>
       </c>
       <c r="P18" s="56" t="s">
-        <v>2668</v>
+        <v>2667</v>
       </c>
       <c r="Q18" s="2"/>
     </row>
@@ -16011,13 +16002,13 @@
         <v>2420</v>
       </c>
       <c r="K19" s="56" t="s">
-        <v>2677</v>
+        <v>2676</v>
       </c>
       <c r="L19" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M19" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N19" s="56" t="s">
         <v>160</v>
@@ -16054,13 +16045,13 @@
       </c>
       <c r="J20" s="56"/>
       <c r="K20" s="56" t="s">
-        <v>2677</v>
+        <v>2676</v>
       </c>
       <c r="L20" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M20" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N20" s="56" t="s">
         <v>166</v>
@@ -16099,13 +16090,13 @@
         <v>2421</v>
       </c>
       <c r="K21" s="56" t="s">
-        <v>2677</v>
+        <v>2676</v>
       </c>
       <c r="L21" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M21" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N21" s="56" t="s">
         <v>172</v>
@@ -16144,16 +16135,16 @@
         <v>178</v>
       </c>
       <c r="K22" s="56" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="L22" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M22" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N22" s="102" t="s">
-        <v>2457</v>
+        <v>2456</v>
       </c>
       <c r="O22" s="56"/>
       <c r="P22" s="58"/>
@@ -16192,10 +16183,10 @@
         <v>185</v>
       </c>
       <c r="L23" s="101" t="s">
-        <v>2507</v>
+        <v>2506</v>
       </c>
       <c r="M23" s="102" t="s">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="N23" s="56" t="s">
         <v>185</v>
@@ -16236,13 +16227,13 @@
         <v>2422</v>
       </c>
       <c r="K24" s="56" t="s">
-        <v>2678</v>
+        <v>2677</v>
       </c>
       <c r="L24" s="101" t="s">
-        <v>2499</v>
+        <v>2498</v>
       </c>
       <c r="M24" s="102" t="s">
-        <v>2508</v>
+        <v>2507</v>
       </c>
       <c r="N24" s="102" t="s">
         <v>191</v>
@@ -16281,22 +16272,22 @@
       </c>
       <c r="J25" s="56"/>
       <c r="K25" s="56" t="s">
-        <v>2679</v>
+        <v>2678</v>
       </c>
       <c r="L25" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M25" s="102" t="s">
-        <v>2501</v>
+        <v>2500</v>
       </c>
       <c r="N25" s="102" t="s">
-        <v>2546</v>
+        <v>2545</v>
       </c>
       <c r="O25" s="102" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
       <c r="P25" s="102" t="s">
-        <v>2664</v>
+        <v>2663</v>
       </c>
       <c r="Q25" s="2"/>
     </row>
@@ -16333,13 +16324,13 @@
         <v>204</v>
       </c>
       <c r="L26" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M26" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N26" s="102" t="s">
-        <v>2460</v>
+        <v>2459</v>
       </c>
       <c r="O26" s="102"/>
       <c r="P26" s="58"/>
@@ -16377,7 +16368,7 @@
         <v>210</v>
       </c>
       <c r="K27" s="56" t="s">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="L27" s="95" t="s">
         <v>211</v>
@@ -16386,13 +16377,13 @@
         <v>212</v>
       </c>
       <c r="N27" s="96" t="s">
-        <v>2696</v>
+        <v>2695</v>
       </c>
       <c r="O27" s="96" t="s">
         <v>213</v>
       </c>
       <c r="P27" s="96" t="s">
-        <v>2663</v>
+        <v>2662</v>
       </c>
       <c r="Q27" s="2"/>
     </row>
@@ -16424,13 +16415,13 @@
       </c>
       <c r="J28" s="56"/>
       <c r="K28" s="56" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="L28" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M28" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N28" s="102" t="s">
         <v>219</v>
@@ -16467,13 +16458,13 @@
       </c>
       <c r="J29" s="56"/>
       <c r="K29" s="56" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="L29" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M29" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N29" s="56" t="s">
         <v>225</v>
@@ -16512,13 +16503,13 @@
         <v>231</v>
       </c>
       <c r="K30" s="56" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="L30" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M30" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N30" s="56" t="s">
         <v>232</v>
@@ -16560,10 +16551,10 @@
         <v>239</v>
       </c>
       <c r="L31" s="101" t="s">
-        <v>2507</v>
+        <v>2506</v>
       </c>
       <c r="M31" s="102" t="s">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="N31" s="102" t="s">
         <v>240</v>
@@ -16602,13 +16593,13 @@
         <v>245</v>
       </c>
       <c r="K32" s="56" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="L32" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M32" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N32" s="56" t="s">
         <v>246</v>
@@ -16645,13 +16636,13 @@
       </c>
       <c r="J33" s="56"/>
       <c r="K33" s="56" t="s">
-        <v>2677</v>
+        <v>2676</v>
       </c>
       <c r="L33" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M33" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N33" s="56" t="s">
         <v>252</v>
@@ -16690,19 +16681,19 @@
         <v>257</v>
       </c>
       <c r="K34" s="104" t="s">
-        <v>2694</v>
+        <v>2693</v>
       </c>
       <c r="L34" s="101" t="s">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="M34" s="55" t="s">
         <v>212</v>
       </c>
       <c r="N34" s="55" t="s">
-        <v>2695</v>
+        <v>2694</v>
       </c>
       <c r="O34" s="56" t="s">
-        <v>2693</v>
+        <v>2692</v>
       </c>
       <c r="P34" s="58"/>
       <c r="Q34" s="2"/>
@@ -16739,13 +16730,13 @@
         <v>263</v>
       </c>
       <c r="K35" s="56" t="s">
-        <v>2682</v>
+        <v>2681</v>
       </c>
       <c r="L35" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M35" s="102" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="N35" s="56" t="s">
         <v>264</v>
@@ -16786,19 +16777,19 @@
         <v>2424</v>
       </c>
       <c r="K36" s="56" t="s">
-        <v>2683</v>
+        <v>2682</v>
       </c>
       <c r="L36" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M36" s="102" t="s">
-        <v>2509</v>
+        <v>2508</v>
       </c>
       <c r="N36" s="102" t="s">
-        <v>2461</v>
+        <v>2460</v>
       </c>
       <c r="O36" s="56" t="s">
-        <v>2467</v>
+        <v>2466</v>
       </c>
       <c r="P36" s="96"/>
       <c r="Q36" s="74"/>
@@ -16835,19 +16826,19 @@
         <v>271</v>
       </c>
       <c r="K37" s="56" t="s">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="L37" s="101" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="M37" s="102" t="s">
-        <v>2509</v>
+        <v>2508</v>
       </c>
       <c r="N37" s="102" t="s">
         <v>278</v>
       </c>
       <c r="O37" s="56" t="s">
-        <v>2468</v>
+        <v>2467</v>
       </c>
       <c r="P37" s="96"/>
       <c r="Q37" s="74"/>
@@ -16884,7 +16875,7 @@
         <v>283</v>
       </c>
       <c r="K38" s="56" t="s">
-        <v>2685</v>
+        <v>2684</v>
       </c>
       <c r="L38" s="101" t="s">
         <v>284</v>
@@ -16933,22 +16924,22 @@
         <v>2425</v>
       </c>
       <c r="K39" s="56" t="s">
-        <v>2686</v>
+        <v>2685</v>
       </c>
       <c r="L39" s="101" t="s">
-        <v>2515</v>
+        <v>2514</v>
       </c>
       <c r="M39" s="102" t="s">
-        <v>2510</v>
+        <v>2509</v>
       </c>
       <c r="N39" s="114" t="s">
         <v>293</v>
       </c>
       <c r="O39" s="114" t="s">
+        <v>2686</v>
+      </c>
+      <c r="P39" s="56" t="s">
         <v>2687</v>
-      </c>
-      <c r="P39" s="56" t="s">
-        <v>2688</v>
       </c>
       <c r="Q39" s="2"/>
     </row>
@@ -16976,16 +16967,16 @@
         <v>33</v>
       </c>
       <c r="I40" s="56" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
       <c r="J40" s="56" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="K40" s="96" t="s">
         <v>298</v>
       </c>
       <c r="L40" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M40" s="102" t="s">
         <v>300</v>
@@ -16994,7 +16985,7 @@
         <v>301</v>
       </c>
       <c r="O40" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P40" s="58"/>
       <c r="Q40" s="75"/>
@@ -17030,7 +17021,7 @@
         <v>298</v>
       </c>
       <c r="L41" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M41" s="102" t="s">
         <v>300</v>
@@ -17039,7 +17030,7 @@
         <v>301</v>
       </c>
       <c r="O41" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P41" s="58"/>
       <c r="Q41" s="75"/>
@@ -17075,7 +17066,7 @@
         <v>298</v>
       </c>
       <c r="L42" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M42" s="102" t="s">
         <v>300</v>
@@ -17084,7 +17075,7 @@
         <v>301</v>
       </c>
       <c r="O42" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P42" s="58"/>
       <c r="Q42" s="2"/>
@@ -17120,7 +17111,7 @@
         <v>298</v>
       </c>
       <c r="L43" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M43" s="102" t="s">
         <v>300</v>
@@ -17129,7 +17120,7 @@
         <v>301</v>
       </c>
       <c r="O43" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P43" s="58"/>
       <c r="Q43" s="2"/>
@@ -17174,7 +17165,7 @@
         <v>301</v>
       </c>
       <c r="O44" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P44" s="58"/>
       <c r="Q44" s="2"/>
@@ -17212,7 +17203,7 @@
         <v>298</v>
       </c>
       <c r="L45" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M45" s="102" t="s">
         <v>300</v>
@@ -17221,7 +17212,7 @@
         <v>301</v>
       </c>
       <c r="O45" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P45" s="58"/>
       <c r="Q45" s="2"/>
@@ -17257,7 +17248,7 @@
         <v>298</v>
       </c>
       <c r="L46" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M46" s="102" t="s">
         <v>300</v>
@@ -17266,7 +17257,7 @@
         <v>301</v>
       </c>
       <c r="O46" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P46" s="58"/>
       <c r="Q46" s="2"/>
@@ -17302,7 +17293,7 @@
         <v>298</v>
       </c>
       <c r="L47" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M47" s="102" t="s">
         <v>300</v>
@@ -17311,7 +17302,7 @@
         <v>301</v>
       </c>
       <c r="O47" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P47" s="58"/>
       <c r="Q47" s="2"/>
@@ -17347,7 +17338,7 @@
         <v>298</v>
       </c>
       <c r="L48" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M48" s="102" t="s">
         <v>300</v>
@@ -17356,7 +17347,7 @@
         <v>301</v>
       </c>
       <c r="O48" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P48" s="58"/>
       <c r="Q48" s="2"/>
@@ -17392,7 +17383,7 @@
         <v>298</v>
       </c>
       <c r="L49" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M49" s="102" t="s">
         <v>300</v>
@@ -17401,7 +17392,7 @@
         <v>301</v>
       </c>
       <c r="O49" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P49" s="58"/>
       <c r="Q49" s="2"/>
@@ -17437,7 +17428,7 @@
         <v>298</v>
       </c>
       <c r="L50" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M50" s="102" t="s">
         <v>300</v>
@@ -17446,7 +17437,7 @@
         <v>301</v>
       </c>
       <c r="O50" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P50" s="58"/>
       <c r="Q50" s="2"/>
@@ -17482,7 +17473,7 @@
         <v>298</v>
       </c>
       <c r="L51" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M51" s="102" t="s">
         <v>300</v>
@@ -17491,7 +17482,7 @@
         <v>301</v>
       </c>
       <c r="O51" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P51" s="58"/>
       <c r="Q51" s="2"/>
@@ -17527,7 +17518,7 @@
         <v>298</v>
       </c>
       <c r="L52" s="95" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
       <c r="M52" s="102" t="s">
         <v>300</v>
@@ -17536,7 +17527,7 @@
         <v>301</v>
       </c>
       <c r="O52" s="96" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="P52" s="58"/>
       <c r="Q52" s="2"/>
@@ -17572,7 +17563,7 @@
         <v>340</v>
       </c>
       <c r="L53" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M53" s="56" t="s">
         <v>341</v>
@@ -17617,7 +17608,7 @@
         <v>340</v>
       </c>
       <c r="L54" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M54" s="56" t="s">
         <v>341</v>
@@ -17662,7 +17653,7 @@
         <v>340</v>
       </c>
       <c r="L55" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M55" s="56" t="s">
         <v>341</v>
@@ -17707,7 +17698,7 @@
         <v>340</v>
       </c>
       <c r="L56" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M56" s="56" t="s">
         <v>341</v>
@@ -17750,7 +17741,7 @@
         <v>340</v>
       </c>
       <c r="L57" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M57" s="56" t="s">
         <v>341</v>
@@ -17759,7 +17750,7 @@
         <v>342</v>
       </c>
       <c r="O57" s="56" t="s">
-        <v>2470</v>
+        <v>2469</v>
       </c>
       <c r="P57" s="58"/>
       <c r="Q57" s="2"/>
@@ -17795,7 +17786,7 @@
         <v>340</v>
       </c>
       <c r="L58" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M58" s="56" t="s">
         <v>341</v>
@@ -17838,7 +17829,7 @@
         <v>340</v>
       </c>
       <c r="L59" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M59" s="56" t="s">
         <v>341</v>
@@ -17881,7 +17872,7 @@
         <v>340</v>
       </c>
       <c r="L60" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M60" s="56" t="s">
         <v>341</v>
@@ -17924,7 +17915,7 @@
         <v>340</v>
       </c>
       <c r="L61" s="95" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
       <c r="M61" s="56" t="s">
         <v>341</v>
@@ -17961,16 +17952,16 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15.75">
       <c r="A1" s="64" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
       <c r="B1" s="64" t="s">
-        <v>2570</v>
+        <v>2569</v>
       </c>
       <c r="C1" s="84" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
       <c r="D1" s="84" t="s">
-        <v>2559</v>
+        <v>2558</v>
       </c>
       <c r="E1" s="84" t="s">
         <v>386</v>
@@ -17987,13 +17978,13 @@
         <v>2452</v>
       </c>
       <c r="C2" s="86" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E2" s="86" t="s">
-        <v>2520</v>
+        <v>2519</v>
       </c>
       <c r="F2" s="85" t="s">
         <v>2444</v>
@@ -18007,13 +17998,13 @@
         <v>2429</v>
       </c>
       <c r="C3" s="86" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>2558</v>
+        <v>2557</v>
       </c>
       <c r="E3" s="85" t="s">
-        <v>2521</v>
+        <v>2520</v>
       </c>
       <c r="F3" s="85" t="s">
         <v>2445</v>
@@ -18027,31 +18018,31 @@
         <v>2429</v>
       </c>
       <c r="C4" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D4" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E4" s="86" t="s">
-        <v>2522</v>
+        <v>2521</v>
       </c>
       <c r="F4" s="86"/>
     </row>
     <row r="5" spans="1:6" ht="15.75">
       <c r="A5" s="8" t="s">
-        <v>2488</v>
+        <v>2487</v>
       </c>
       <c r="B5" s="86" t="s">
         <v>2452</v>
       </c>
       <c r="C5" s="86" t="s">
-        <v>2551</v>
+        <v>2550</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E5" s="86" t="s">
-        <v>2523</v>
+        <v>2522</v>
       </c>
       <c r="F5" s="86"/>
     </row>
@@ -18063,16 +18054,16 @@
         <v>2429</v>
       </c>
       <c r="C6" s="86" t="s">
-        <v>2556</v>
+        <v>2555</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>2567</v>
+        <v>2566</v>
       </c>
       <c r="E6" s="85" t="s">
-        <v>2524</v>
+        <v>2523</v>
       </c>
       <c r="F6" s="85" t="s">
-        <v>2560</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="126">
@@ -18083,13 +18074,13 @@
         <v>2429</v>
       </c>
       <c r="C7" s="86" t="s">
-        <v>2556</v>
+        <v>2555</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>2567</v>
+        <v>2566</v>
       </c>
       <c r="E7" s="86" t="s">
-        <v>2525</v>
+        <v>2524</v>
       </c>
       <c r="F7" s="85" t="s">
         <v>2453</v>
@@ -18103,13 +18094,13 @@
         <v>2429</v>
       </c>
       <c r="C8" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D8" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E8" t="s">
-        <v>2519</v>
+        <v>2518</v>
       </c>
       <c r="F8" s="86"/>
     </row>
@@ -18121,13 +18112,13 @@
         <v>2429</v>
       </c>
       <c r="C9" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E9" t="s">
-        <v>2491</v>
+        <v>2490</v>
       </c>
       <c r="F9" s="86"/>
     </row>
@@ -18139,16 +18130,16 @@
         <v>2429</v>
       </c>
       <c r="C10" s="86" t="s">
-        <v>2552</v>
+        <v>2551</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E10" t="s">
-        <v>2492</v>
+        <v>2491</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>2561</v>
+        <v>2560</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15.75">
@@ -18159,16 +18150,16 @@
         <v>2429</v>
       </c>
       <c r="C11" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D11" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E11" t="s">
+        <v>2492</v>
+      </c>
+      <c r="F11" t="s">
         <v>2493</v>
-      </c>
-      <c r="F11" t="s">
-        <v>2494</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="30">
@@ -18179,16 +18170,16 @@
         <v>2429</v>
       </c>
       <c r="C12" s="86" t="s">
-        <v>2551</v>
+        <v>2550</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>2558</v>
+        <v>2557</v>
       </c>
       <c r="E12" t="s">
-        <v>2535</v>
+        <v>2534</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>2562</v>
+        <v>2561</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15.75">
@@ -18199,13 +18190,13 @@
         <v>2429</v>
       </c>
       <c r="C13" s="86" t="s">
-        <v>2568</v>
+        <v>2567</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E13" t="s">
-        <v>2495</v>
+        <v>2494</v>
       </c>
       <c r="F13" s="86"/>
     </row>
@@ -18217,16 +18208,16 @@
         <v>2429</v>
       </c>
       <c r="C14" s="86" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>2569</v>
+        <v>2568</v>
       </c>
       <c r="E14" t="s">
-        <v>2534</v>
+        <v>2533</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>2563</v>
+        <v>2562</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="15.75">
@@ -18237,13 +18228,13 @@
         <v>2429</v>
       </c>
       <c r="C15" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D15" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E15" t="s">
-        <v>2533</v>
+        <v>2532</v>
       </c>
       <c r="F15" s="86"/>
     </row>
@@ -18255,16 +18246,16 @@
         <v>2429</v>
       </c>
       <c r="C16" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D16" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E16" t="s">
-        <v>2532</v>
+        <v>2531</v>
       </c>
       <c r="F16" s="85" t="s">
-        <v>2564</v>
+        <v>2563</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15.75">
@@ -18275,19 +18266,19 @@
         <v>2429</v>
       </c>
       <c r="C17" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D17" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E17" t="s">
-        <v>2531</v>
+        <v>2530</v>
       </c>
       <c r="F17" s="86"/>
     </row>
     <row r="18" spans="1:7" ht="15.75">
       <c r="A18" s="8" t="s">
-        <v>2489</v>
+        <v>2488</v>
       </c>
       <c r="B18" s="86" t="s">
         <v>2452</v>
@@ -18296,18 +18287,18 @@
         <v>2242</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E18" s="86" t="s">
-        <v>2575</v>
+        <v>2574</v>
       </c>
       <c r="F18" s="86" t="s">
-        <v>2476</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="15.75">
       <c r="A19" s="8" t="s">
-        <v>2490</v>
+        <v>2489</v>
       </c>
       <c r="B19" s="86" t="s">
         <v>2452</v>
@@ -18316,149 +18307,149 @@
         <v>2242</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E19" s="86" t="s">
-        <v>2576</v>
+        <v>2575</v>
       </c>
       <c r="F19" s="86"/>
     </row>
     <row r="20" spans="1:7" ht="47.25">
       <c r="A20" s="8" t="s">
-        <v>2487</v>
+        <v>2486</v>
       </c>
       <c r="B20" s="86" t="s">
-        <v>2473</v>
+        <v>2472</v>
       </c>
       <c r="C20" s="86" t="s">
-        <v>2556</v>
+        <v>2555</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>2571</v>
+        <v>2570</v>
       </c>
       <c r="E20" s="86" t="s">
-        <v>2577</v>
+        <v>2576</v>
       </c>
       <c r="F20" s="85" t="s">
-        <v>2565</v>
+        <v>2564</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15.75">
       <c r="A21" s="8" t="s">
-        <v>2486</v>
+        <v>2485</v>
       </c>
       <c r="B21" s="86" t="s">
-        <v>2474</v>
+        <v>2473</v>
       </c>
       <c r="C21" s="86" t="s">
+        <v>2555</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>2556</v>
       </c>
-      <c r="D21" s="8" t="s">
-        <v>2557</v>
-      </c>
       <c r="E21" s="86" t="s">
-        <v>2526</v>
+        <v>2525</v>
       </c>
       <c r="F21" s="86"/>
     </row>
     <row r="22" spans="1:7" ht="15.75">
       <c r="A22" s="8" t="s">
-        <v>2483</v>
+        <v>2482</v>
       </c>
       <c r="B22" s="86" t="s">
         <v>296</v>
       </c>
       <c r="C22" s="86" t="s">
-        <v>2553</v>
+        <v>2552</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E22" s="86" t="s">
-        <v>2529</v>
+        <v>2528</v>
       </c>
       <c r="F22" s="86" t="s">
-        <v>2475</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="31.5">
       <c r="A23" s="8" t="s">
-        <v>2484</v>
+        <v>2483</v>
       </c>
       <c r="B23" s="86" t="s">
         <v>296</v>
       </c>
       <c r="C23" s="86" t="s">
-        <v>2554</v>
+        <v>2553</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E23" s="85" t="s">
-        <v>2528</v>
+        <v>2527</v>
       </c>
       <c r="F23" s="86" t="s">
-        <v>2475</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75">
       <c r="A24" s="8" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
       <c r="B24" s="86" t="s">
         <v>296</v>
       </c>
       <c r="C24" s="86" t="s">
-        <v>2555</v>
+        <v>2554</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
       <c r="E24" s="86" t="s">
-        <v>2527</v>
+        <v>2526</v>
       </c>
       <c r="F24" s="86" t="s">
-        <v>2475</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="15.75">
       <c r="A25" s="8" t="s">
+        <v>2478</v>
+      </c>
+      <c r="B25" s="86" t="s">
+        <v>2476</v>
+      </c>
+      <c r="C25" s="86" t="s">
+        <v>2571</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>2556</v>
+      </c>
+      <c r="E25" s="86" t="s">
+        <v>2529</v>
+      </c>
+      <c r="F25" s="86" t="s">
         <v>2479</v>
-      </c>
-      <c r="B25" s="86" t="s">
-        <v>2477</v>
-      </c>
-      <c r="C25" s="86" t="s">
-        <v>2572</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>2557</v>
-      </c>
-      <c r="E25" s="86" t="s">
-        <v>2530</v>
-      </c>
-      <c r="F25" s="86" t="s">
-        <v>2480</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="15.75">
       <c r="A26" s="8" t="s">
+        <v>2480</v>
+      </c>
+      <c r="B26" s="86" t="s">
+        <v>2477</v>
+      </c>
+      <c r="C26" s="86" t="s">
+        <v>2477</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>2572</v>
+      </c>
+      <c r="E26" s="86" t="s">
+        <v>2535</v>
+      </c>
+      <c r="F26" s="86" t="s">
         <v>2481</v>
-      </c>
-      <c r="B26" s="86" t="s">
-        <v>2478</v>
-      </c>
-      <c r="C26" s="86" t="s">
-        <v>2478</v>
-      </c>
-      <c r="D26" s="8" t="s">
-        <v>2573</v>
-      </c>
-      <c r="E26" s="86" t="s">
-        <v>2536</v>
-      </c>
-      <c r="F26" s="86" t="s">
-        <v>2482</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="47.25">
@@ -18469,14 +18460,14 @@
         <v>2429</v>
       </c>
       <c r="C27" s="86" t="s">
-        <v>2574</v>
+        <v>2573</v>
       </c>
       <c r="D27" s="86"/>
       <c r="E27" s="85" t="s">
-        <v>2537</v>
+        <v>2536</v>
       </c>
       <c r="F27" s="85" t="s">
-        <v>2566</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="15.75">
@@ -18487,11 +18478,11 @@
         <v>2451</v>
       </c>
       <c r="C28" s="86" t="s">
-        <v>2574</v>
+        <v>2573</v>
       </c>
       <c r="D28" s="86"/>
       <c r="E28" s="86" t="s">
-        <v>2538</v>
+        <v>2537</v>
       </c>
       <c r="F28" s="86"/>
     </row>
@@ -18503,11 +18494,11 @@
         <v>2451</v>
       </c>
       <c r="C29" s="86" t="s">
-        <v>2574</v>
+        <v>2573</v>
       </c>
       <c r="D29" s="86"/>
       <c r="E29" s="86" t="s">
-        <v>2539</v>
+        <v>2538</v>
       </c>
       <c r="F29" s="86"/>
     </row>
@@ -18597,19 +18588,19 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>2582</v>
+        <v>2581</v>
       </c>
       <c r="B1" t="s">
-        <v>2589</v>
+        <v>2588</v>
       </c>
       <c r="C1" t="s">
+        <v>2577</v>
+      </c>
+      <c r="D1" t="s">
         <v>2578</v>
       </c>
-      <c r="D1" t="s">
-        <v>2579</v>
-      </c>
       <c r="E1" t="s">
-        <v>2587</v>
+        <v>2586</v>
       </c>
       <c r="F1" t="s">
         <v>2327</v>
@@ -18617,532 +18608,532 @@
     </row>
     <row r="2" spans="1:6" ht="30">
       <c r="A2" s="8" t="s">
-        <v>2584</v>
+        <v>2583</v>
       </c>
       <c r="B2" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C2" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="D2" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>2652</v>
+        <v>2651</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="8" t="s">
-        <v>2583</v>
+        <v>2582</v>
       </c>
       <c r="B3" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C3" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="D3" s="91" t="s">
-        <v>2620</v>
+        <v>2619</v>
       </c>
       <c r="E3" t="s">
-        <v>2653</v>
+        <v>2652</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="8" t="s">
-        <v>2585</v>
+        <v>2584</v>
       </c>
       <c r="B4" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C4" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="D4" s="91" t="s">
-        <v>2626</v>
+        <v>2625</v>
       </c>
       <c r="E4" t="s">
-        <v>2654</v>
+        <v>2653</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="8" t="s">
-        <v>2586</v>
+        <v>2585</v>
       </c>
       <c r="B5" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C5" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="D5" s="91" t="s">
-        <v>2620</v>
+        <v>2619</v>
       </c>
       <c r="E5" t="s">
-        <v>2655</v>
+        <v>2654</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="30">
       <c r="A6" s="8" t="s">
-        <v>2588</v>
+        <v>2587</v>
       </c>
       <c r="B6" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C6" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="D6" s="91" t="s">
-        <v>2620</v>
+        <v>2619</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>2657</v>
+        <v>2656</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="8" t="s">
-        <v>2593</v>
+        <v>2592</v>
       </c>
       <c r="B7" s="90" t="s">
-        <v>2592</v>
+        <v>2591</v>
       </c>
       <c r="C7" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="D7" s="91" t="s">
-        <v>2620</v>
+        <v>2619</v>
       </c>
       <c r="E7" t="s">
-        <v>2656</v>
+        <v>2655</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="45">
       <c r="A8" s="8" t="s">
-        <v>2594</v>
+        <v>2593</v>
       </c>
       <c r="B8" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C8" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D8" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>2627</v>
+        <v>2626</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>2651</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="8" t="s">
-        <v>2595</v>
+        <v>2594</v>
       </c>
       <c r="B9" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C9" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D9" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>2628</v>
+        <v>2627</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="8" t="s">
-        <v>2596</v>
+        <v>2595</v>
       </c>
       <c r="B10" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C10" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D10" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>2629</v>
+        <v>2628</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="8" t="s">
-        <v>2597</v>
+        <v>2596</v>
       </c>
       <c r="B11" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C11" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D11" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>2630</v>
+        <v>2629</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="60">
       <c r="A12" s="8" t="s">
+        <v>2597</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2589</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2579</v>
+      </c>
+      <c r="D12" t="s">
         <v>2598</v>
       </c>
-      <c r="B12" t="s">
-        <v>2590</v>
-      </c>
-      <c r="C12" t="s">
-        <v>2580</v>
-      </c>
-      <c r="D12" t="s">
-        <v>2599</v>
-      </c>
       <c r="E12" s="10" t="s">
-        <v>2631</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="60">
       <c r="A13" s="8" t="s">
-        <v>2600</v>
+        <v>2599</v>
       </c>
       <c r="B13" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C13" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D13" t="s">
-        <v>2621</v>
+        <v>2620</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>2631</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="30">
       <c r="A14" s="8" t="s">
-        <v>2601</v>
+        <v>2600</v>
       </c>
       <c r="B14" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C14" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D14" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>2632</v>
+        <v>2631</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="8" t="s">
-        <v>2602</v>
+        <v>2601</v>
       </c>
       <c r="B15" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C15" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D15" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>2633</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="45">
       <c r="A16" s="8" t="s">
-        <v>2603</v>
+        <v>2602</v>
       </c>
       <c r="B16" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C16" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D16" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>2634</v>
+        <v>2633</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="8" t="s">
-        <v>2604</v>
+        <v>2603</v>
       </c>
       <c r="B17" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C17" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D17" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>2635</v>
+        <v>2634</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30">
       <c r="A18" s="8" t="s">
-        <v>2605</v>
+        <v>2604</v>
       </c>
       <c r="B18" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C18" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D18" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>2636</v>
+        <v>2635</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30">
       <c r="A19" s="8" t="s">
-        <v>2606</v>
+        <v>2605</v>
       </c>
       <c r="B19" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C19" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D19" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>2637</v>
+        <v>2636</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="8" t="s">
-        <v>2607</v>
+        <v>2606</v>
       </c>
       <c r="B20" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C20" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D20" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>2638</v>
+        <v>2637</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="8" t="s">
-        <v>2608</v>
+        <v>2607</v>
       </c>
       <c r="B21" s="90" t="s">
-        <v>2592</v>
+        <v>2591</v>
       </c>
       <c r="C21" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D21" s="91" t="s">
-        <v>2620</v>
+        <v>2619</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>2639</v>
+        <v>2638</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="8" t="s">
-        <v>2609</v>
+        <v>2608</v>
       </c>
       <c r="B22" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C22" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D22" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>2640</v>
+        <v>2639</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="8" t="s">
-        <v>2610</v>
+        <v>2609</v>
       </c>
       <c r="B23" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C23" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D23" t="s">
-        <v>2599</v>
+        <v>2598</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>2641</v>
+        <v>2640</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="45">
       <c r="A24" s="8" t="s">
-        <v>2611</v>
+        <v>2610</v>
       </c>
       <c r="B24" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C24" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D24" t="s">
-        <v>2622</v>
+        <v>2621</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>2642</v>
+        <v>2641</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="8" t="s">
-        <v>2612</v>
+        <v>2611</v>
       </c>
       <c r="B25" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C25" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D25" t="s">
-        <v>2622</v>
+        <v>2621</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>2643</v>
+        <v>2642</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="45">
       <c r="A26" s="8" t="s">
-        <v>2613</v>
+        <v>2612</v>
       </c>
       <c r="B26" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C26" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D26" t="s">
-        <v>2658</v>
+        <v>2657</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>2644</v>
+        <v>2643</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="8" t="s">
-        <v>2614</v>
+        <v>2613</v>
       </c>
       <c r="B27" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C27" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D27" s="91" t="s">
-        <v>2626</v>
+        <v>2625</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>2645</v>
+        <v>2644</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="30">
       <c r="A28" s="8" t="s">
-        <v>2615</v>
+        <v>2614</v>
       </c>
       <c r="B28" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C28" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D28" t="s">
-        <v>2622</v>
+        <v>2621</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>2646</v>
+        <v>2645</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="8" t="s">
-        <v>2616</v>
+        <v>2615</v>
       </c>
       <c r="B29" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C29" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D29" t="s">
-        <v>2623</v>
+        <v>2622</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>2647</v>
+        <v>2646</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="8" t="s">
-        <v>2617</v>
+        <v>2616</v>
       </c>
       <c r="B30" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
       <c r="C30" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D30" t="s">
-        <v>2625</v>
+        <v>2624</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>2648</v>
+        <v>2647</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="8" t="s">
-        <v>2618</v>
+        <v>2617</v>
       </c>
       <c r="B31" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C31" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D31" t="s">
-        <v>2622</v>
+        <v>2621</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>2649</v>
+        <v>2648</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="60">
       <c r="A32" s="8" t="s">
-        <v>2619</v>
+        <v>2618</v>
       </c>
       <c r="B32" t="s">
-        <v>2591</v>
+        <v>2590</v>
       </c>
       <c r="C32" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="D32" t="s">
-        <v>2624</v>
+        <v>2623</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>2650</v>
+        <v>2649</v>
       </c>
     </row>
   </sheetData>
@@ -25317,10 +25308,10 @@
       <c r="E2" s="43" t="s">
         <v>1194</v>
       </c>
-      <c r="F2" s="119" t="s">
+      <c r="F2" s="120" t="s">
         <v>1195</v>
       </c>
-      <c r="G2" s="119"/>
+      <c r="G2" s="120"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="43"/>
@@ -25394,10 +25385,10 @@
       <c r="E7" s="44" t="s">
         <v>1194</v>
       </c>
-      <c r="F7" s="120" t="s">
+      <c r="F7" s="121" t="s">
         <v>1205</v>
       </c>
-      <c r="G7" s="116"/>
+      <c r="G7" s="117"/>
     </row>
     <row r="8" spans="1:7" s="44" customFormat="1">
       <c r="D8" s="44" t="s">
@@ -25406,8 +25397,8 @@
       <c r="E8" s="44" t="s">
         <v>1199</v>
       </c>
-      <c r="F8" s="120"/>
-      <c r="G8" s="116"/>
+      <c r="F8" s="121"/>
+      <c r="G8" s="117"/>
     </row>
     <row r="9" spans="1:7" s="44" customFormat="1">
       <c r="D9" s="44" t="s">
@@ -25416,8 +25407,8 @@
       <c r="E9" s="44" t="s">
         <v>1201</v>
       </c>
-      <c r="F9" s="120"/>
-      <c r="G9" s="116"/>
+      <c r="F9" s="121"/>
+      <c r="G9" s="117"/>
     </row>
     <row r="10" spans="1:7" s="44" customFormat="1">
       <c r="D10" s="44" t="s">
@@ -25426,8 +25417,8 @@
       <c r="E10" s="44" t="s">
         <v>1203</v>
       </c>
-      <c r="F10" s="120"/>
-      <c r="G10" s="116"/>
+      <c r="F10" s="121"/>
+      <c r="G10" s="117"/>
     </row>
     <row r="11" spans="1:7" s="44" customFormat="1">
       <c r="B11" s="44" t="s">
@@ -25442,8 +25433,8 @@
       <c r="E11" s="44" t="s">
         <v>1194</v>
       </c>
-      <c r="F11" s="120"/>
-      <c r="G11" s="116"/>
+      <c r="F11" s="121"/>
+      <c r="G11" s="117"/>
     </row>
     <row r="12" spans="1:7" s="44" customFormat="1">
       <c r="B12" s="44" t="s">
@@ -25452,8 +25443,8 @@
       <c r="C12" s="44" t="s">
         <v>1207</v>
       </c>
-      <c r="F12" s="120"/>
-      <c r="G12" s="116"/>
+      <c r="F12" s="121"/>
+      <c r="G12" s="117"/>
     </row>
     <row r="13" spans="1:7" s="44" customFormat="1">
       <c r="B13" s="44" t="s">
@@ -25462,8 +25453,8 @@
       <c r="C13" s="44" t="s">
         <v>1209</v>
       </c>
-      <c r="F13" s="120"/>
-      <c r="G13" s="116"/>
+      <c r="F13" s="121"/>
+      <c r="G13" s="117"/>
     </row>
     <row r="14" spans="1:7" s="43" customFormat="1">
       <c r="A14" s="43" t="s">
@@ -25475,7 +25466,7 @@
       <c r="C14" s="43" t="s">
         <v>1197</v>
       </c>
-      <c r="F14" s="121" t="s">
+      <c r="F14" s="122" t="s">
         <v>1211</v>
       </c>
       <c r="G14" s="118" t="s">
@@ -25534,10 +25525,10 @@
       </c>
       <c r="D19" s="44"/>
       <c r="E19" s="44"/>
-      <c r="F19" s="122" t="s">
+      <c r="F19" s="116" t="s">
         <v>1195</v>
       </c>
-      <c r="G19" s="116"/>
+      <c r="G19" s="117"/>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="44"/>
@@ -25549,8 +25540,8 @@
       </c>
       <c r="D20" s="44"/>
       <c r="E20" s="44"/>
-      <c r="F20" s="116"/>
-      <c r="G20" s="116"/>
+      <c r="F20" s="117"/>
+      <c r="G20" s="117"/>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="44"/>
@@ -25562,8 +25553,8 @@
       </c>
       <c r="D21" s="44"/>
       <c r="E21" s="44"/>
-      <c r="F21" s="116"/>
-      <c r="G21" s="116"/>
+      <c r="F21" s="117"/>
+      <c r="G21" s="117"/>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="44"/>
@@ -25575,8 +25566,8 @@
       </c>
       <c r="D22" s="44"/>
       <c r="E22" s="44"/>
-      <c r="F22" s="116"/>
-      <c r="G22" s="116"/>
+      <c r="F22" s="117"/>
+      <c r="G22" s="117"/>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="44"/>
@@ -25588,8 +25579,8 @@
       </c>
       <c r="D23" s="44"/>
       <c r="E23" s="44"/>
-      <c r="F23" s="116"/>
-      <c r="G23" s="116"/>
+      <c r="F23" s="117"/>
+      <c r="G23" s="117"/>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="43" t="s">
@@ -25622,10 +25613,10 @@
       </c>
       <c r="D25" s="44"/>
       <c r="E25" s="44"/>
-      <c r="F25" s="116" t="s">
+      <c r="F25" s="117" t="s">
         <v>1195</v>
       </c>
-      <c r="G25" s="123"/>
+      <c r="G25" s="119"/>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" s="44"/>
@@ -25637,8 +25628,8 @@
       </c>
       <c r="D26" s="44"/>
       <c r="E26" s="44"/>
-      <c r="F26" s="116"/>
-      <c r="G26" s="123"/>
+      <c r="F26" s="117"/>
+      <c r="G26" s="119"/>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="44"/>
@@ -25650,8 +25641,8 @@
       </c>
       <c r="D27" s="44"/>
       <c r="E27" s="44"/>
-      <c r="F27" s="116"/>
-      <c r="G27" s="123"/>
+      <c r="F27" s="117"/>
+      <c r="G27" s="119"/>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="44"/>
@@ -25663,8 +25654,8 @@
       </c>
       <c r="D28" s="44"/>
       <c r="E28" s="44"/>
-      <c r="F28" s="116"/>
-      <c r="G28" s="123"/>
+      <c r="F28" s="117"/>
+      <c r="G28" s="119"/>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" s="44"/>
@@ -25676,8 +25667,8 @@
       </c>
       <c r="D29" s="44"/>
       <c r="E29" s="44"/>
-      <c r="F29" s="116"/>
-      <c r="G29" s="123"/>
+      <c r="F29" s="117"/>
+      <c r="G29" s="119"/>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" s="44"/>
@@ -25689,8 +25680,8 @@
       </c>
       <c r="D30" s="44"/>
       <c r="E30" s="44"/>
-      <c r="F30" s="116"/>
-      <c r="G30" s="123"/>
+      <c r="F30" s="117"/>
+      <c r="G30" s="119"/>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="44"/>
@@ -25702,8 +25693,8 @@
       </c>
       <c r="D31" s="44"/>
       <c r="E31" s="44"/>
-      <c r="F31" s="116"/>
-      <c r="G31" s="123"/>
+      <c r="F31" s="117"/>
+      <c r="G31" s="119"/>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" s="43" t="s">
@@ -26141,10 +26132,10 @@
       </c>
       <c r="D64" s="44"/>
       <c r="E64" s="44"/>
-      <c r="F64" s="116" t="s">
+      <c r="F64" s="117" t="s">
         <v>1306</v>
       </c>
-      <c r="G64" s="116"/>
+      <c r="G64" s="117"/>
     </row>
     <row r="65" spans="1:7">
       <c r="A65" s="44"/>
@@ -26156,8 +26147,8 @@
       <c r="E65" s="44" t="s">
         <v>1308</v>
       </c>
-      <c r="F65" s="116"/>
-      <c r="G65" s="116"/>
+      <c r="F65" s="117"/>
+      <c r="G65" s="117"/>
     </row>
     <row r="66" spans="1:7">
       <c r="A66" s="44"/>
@@ -26169,8 +26160,8 @@
       <c r="E66" s="44" t="s">
         <v>1310</v>
       </c>
-      <c r="F66" s="116"/>
-      <c r="G66" s="116"/>
+      <c r="F66" s="117"/>
+      <c r="G66" s="117"/>
     </row>
     <row r="67" spans="1:7">
       <c r="A67" s="44"/>
@@ -26182,8 +26173,8 @@
       </c>
       <c r="D67" s="44"/>
       <c r="E67" s="44"/>
-      <c r="F67" s="116"/>
-      <c r="G67" s="116"/>
+      <c r="F67" s="117"/>
+      <c r="G67" s="117"/>
     </row>
     <row r="68" spans="1:7">
       <c r="A68" s="44"/>
@@ -26195,8 +26186,8 @@
       <c r="E68" s="44" t="s">
         <v>1314</v>
       </c>
-      <c r="F68" s="116"/>
-      <c r="G68" s="116"/>
+      <c r="F68" s="117"/>
+      <c r="G68" s="117"/>
     </row>
     <row r="69" spans="1:7">
       <c r="A69" s="44"/>
@@ -26212,8 +26203,8 @@
       <c r="E69" s="44" t="s">
         <v>1318</v>
       </c>
-      <c r="F69" s="116"/>
-      <c r="G69" s="116"/>
+      <c r="F69" s="117"/>
+      <c r="G69" s="117"/>
     </row>
     <row r="70" spans="1:7">
       <c r="A70" s="44"/>
@@ -26225,8 +26216,8 @@
       <c r="E70" s="44" t="s">
         <v>1320</v>
       </c>
-      <c r="F70" s="116"/>
-      <c r="G70" s="116"/>
+      <c r="F70" s="117"/>
+      <c r="G70" s="117"/>
     </row>
     <row r="71" spans="1:7">
       <c r="A71" s="44"/>
@@ -26238,8 +26229,8 @@
       <c r="E71" s="44" t="s">
         <v>1322</v>
       </c>
-      <c r="F71" s="116"/>
-      <c r="G71" s="116"/>
+      <c r="F71" s="117"/>
+      <c r="G71" s="117"/>
     </row>
     <row r="72" spans="1:7">
       <c r="A72" s="44"/>
@@ -26251,8 +26242,8 @@
       <c r="E72" s="44" t="s">
         <v>1324</v>
       </c>
-      <c r="F72" s="116"/>
-      <c r="G72" s="116"/>
+      <c r="F72" s="117"/>
+      <c r="G72" s="117"/>
     </row>
     <row r="73" spans="1:7">
       <c r="A73" s="44"/>
@@ -26264,8 +26255,8 @@
       <c r="E73" s="44" t="s">
         <v>1326</v>
       </c>
-      <c r="F73" s="116"/>
-      <c r="G73" s="116"/>
+      <c r="F73" s="117"/>
+      <c r="G73" s="117"/>
     </row>
     <row r="74" spans="1:7">
       <c r="A74" s="44"/>
@@ -26277,8 +26268,8 @@
       </c>
       <c r="D74" s="44"/>
       <c r="E74" s="44"/>
-      <c r="F74" s="116"/>
-      <c r="G74" s="116"/>
+      <c r="F74" s="117"/>
+      <c r="G74" s="117"/>
     </row>
     <row r="75" spans="1:7">
       <c r="A75" s="44"/>
@@ -26290,8 +26281,8 @@
       <c r="E75" s="44" t="s">
         <v>1330</v>
       </c>
-      <c r="F75" s="116"/>
-      <c r="G75" s="116"/>
+      <c r="F75" s="117"/>
+      <c r="G75" s="117"/>
     </row>
     <row r="76" spans="1:7">
       <c r="A76" s="44"/>
@@ -26307,8 +26298,8 @@
       <c r="E76" s="44" t="s">
         <v>1334</v>
       </c>
-      <c r="F76" s="116"/>
-      <c r="G76" s="116"/>
+      <c r="F76" s="117"/>
+      <c r="G76" s="117"/>
     </row>
     <row r="77" spans="1:7">
       <c r="A77" s="44"/>
@@ -26320,8 +26311,8 @@
       <c r="E77" s="44" t="s">
         <v>1336</v>
       </c>
-      <c r="F77" s="116"/>
-      <c r="G77" s="116"/>
+      <c r="F77" s="117"/>
+      <c r="G77" s="117"/>
     </row>
     <row r="78" spans="1:7">
       <c r="A78" s="44"/>
@@ -26333,8 +26324,8 @@
       <c r="E78" s="44" t="s">
         <v>1338</v>
       </c>
-      <c r="F78" s="116"/>
-      <c r="G78" s="116"/>
+      <c r="F78" s="117"/>
+      <c r="G78" s="117"/>
     </row>
     <row r="79" spans="1:7">
       <c r="A79" s="44"/>
@@ -26346,8 +26337,8 @@
       <c r="E79" s="44" t="s">
         <v>1340</v>
       </c>
-      <c r="F79" s="116"/>
-      <c r="G79" s="116"/>
+      <c r="F79" s="117"/>
+      <c r="G79" s="117"/>
     </row>
     <row r="80" spans="1:7">
       <c r="A80" s="44"/>
@@ -26359,8 +26350,8 @@
       <c r="E80" s="44" t="s">
         <v>1342</v>
       </c>
-      <c r="F80" s="116"/>
-      <c r="G80" s="116"/>
+      <c r="F80" s="117"/>
+      <c r="G80" s="117"/>
     </row>
     <row r="81" spans="1:7">
       <c r="A81" s="44"/>
@@ -26376,8 +26367,8 @@
       <c r="E81" s="44" t="s">
         <v>1346</v>
       </c>
-      <c r="F81" s="116"/>
-      <c r="G81" s="116"/>
+      <c r="F81" s="117"/>
+      <c r="G81" s="117"/>
     </row>
     <row r="82" spans="1:7">
       <c r="A82" s="44"/>
@@ -26389,8 +26380,8 @@
       <c r="E82" s="44" t="s">
         <v>1348</v>
       </c>
-      <c r="F82" s="116"/>
-      <c r="G82" s="116"/>
+      <c r="F82" s="117"/>
+      <c r="G82" s="117"/>
     </row>
     <row r="83" spans="1:7">
       <c r="A83" s="44"/>
@@ -26402,8 +26393,8 @@
       <c r="E83" s="44" t="s">
         <v>1350</v>
       </c>
-      <c r="F83" s="116"/>
-      <c r="G83" s="116"/>
+      <c r="F83" s="117"/>
+      <c r="G83" s="117"/>
     </row>
     <row r="84" spans="1:7">
       <c r="A84" s="44"/>
@@ -26415,8 +26406,8 @@
       </c>
       <c r="D84" s="44"/>
       <c r="E84" s="44"/>
-      <c r="F84" s="116"/>
-      <c r="G84" s="116"/>
+      <c r="F84" s="117"/>
+      <c r="G84" s="117"/>
     </row>
     <row r="85" spans="1:7">
       <c r="A85" s="44"/>
@@ -26428,8 +26419,8 @@
       <c r="E85" s="44" t="s">
         <v>1354</v>
       </c>
-      <c r="F85" s="116"/>
-      <c r="G85" s="116"/>
+      <c r="F85" s="117"/>
+      <c r="G85" s="117"/>
     </row>
     <row r="86" spans="1:7">
       <c r="A86" s="44"/>
@@ -26441,8 +26432,8 @@
       <c r="E86" s="44" t="s">
         <v>1356</v>
       </c>
-      <c r="F86" s="116"/>
-      <c r="G86" s="116"/>
+      <c r="F86" s="117"/>
+      <c r="G86" s="117"/>
     </row>
     <row r="87" spans="1:7">
       <c r="A87" s="44"/>
@@ -26454,8 +26445,8 @@
       <c r="E87" s="44" t="s">
         <v>1358</v>
       </c>
-      <c r="F87" s="116"/>
-      <c r="G87" s="116"/>
+      <c r="F87" s="117"/>
+      <c r="G87" s="117"/>
     </row>
     <row r="88" spans="1:7">
       <c r="A88" s="44"/>
@@ -26467,8 +26458,8 @@
       </c>
       <c r="D88" s="44"/>
       <c r="E88" s="44"/>
-      <c r="F88" s="116"/>
-      <c r="G88" s="116"/>
+      <c r="F88" s="117"/>
+      <c r="G88" s="117"/>
     </row>
     <row r="89" spans="1:7">
       <c r="A89" s="43" t="s">
@@ -26499,10 +26490,10 @@
       </c>
       <c r="D90" s="44"/>
       <c r="E90" s="44"/>
-      <c r="F90" s="116" t="s">
+      <c r="F90" s="117" t="s">
         <v>1364</v>
       </c>
-      <c r="G90" s="116"/>
+      <c r="G90" s="117"/>
     </row>
     <row r="91" spans="1:7">
       <c r="A91" s="44"/>
@@ -26514,8 +26505,8 @@
       </c>
       <c r="D91" s="44"/>
       <c r="E91" s="44"/>
-      <c r="F91" s="116"/>
-      <c r="G91" s="116"/>
+      <c r="F91" s="117"/>
+      <c r="G91" s="117"/>
     </row>
     <row r="92" spans="1:7">
       <c r="A92" s="44"/>
@@ -26527,8 +26518,8 @@
       <c r="E92" s="44" t="s">
         <v>1368</v>
       </c>
-      <c r="F92" s="116"/>
-      <c r="G92" s="116"/>
+      <c r="F92" s="117"/>
+      <c r="G92" s="117"/>
     </row>
     <row r="93" spans="1:7">
       <c r="A93" s="44"/>
@@ -26540,8 +26531,8 @@
       </c>
       <c r="D93" s="44"/>
       <c r="E93" s="44"/>
-      <c r="F93" s="116"/>
-      <c r="G93" s="116"/>
+      <c r="F93" s="117"/>
+      <c r="G93" s="117"/>
     </row>
     <row r="94" spans="1:7">
       <c r="A94" s="44"/>
@@ -26553,8 +26544,8 @@
       </c>
       <c r="D94" s="44"/>
       <c r="E94" s="44"/>
-      <c r="F94" s="116"/>
-      <c r="G94" s="116"/>
+      <c r="F94" s="117"/>
+      <c r="G94" s="117"/>
     </row>
     <row r="95" spans="1:7">
       <c r="A95" s="44"/>
@@ -26566,8 +26557,8 @@
       <c r="E95" s="44" t="s">
         <v>1374</v>
       </c>
-      <c r="F95" s="116"/>
-      <c r="G95" s="116"/>
+      <c r="F95" s="117"/>
+      <c r="G95" s="117"/>
     </row>
     <row r="96" spans="1:7">
       <c r="A96" s="44"/>
@@ -26579,8 +26570,8 @@
       <c r="E96" s="44" t="s">
         <v>1376</v>
       </c>
-      <c r="F96" s="116"/>
-      <c r="G96" s="116"/>
+      <c r="F96" s="117"/>
+      <c r="G96" s="117"/>
     </row>
     <row r="97" spans="1:7">
       <c r="A97" s="44"/>
@@ -26592,8 +26583,8 @@
       <c r="E97" s="44" t="s">
         <v>1378</v>
       </c>
-      <c r="F97" s="116"/>
-      <c r="G97" s="116"/>
+      <c r="F97" s="117"/>
+      <c r="G97" s="117"/>
     </row>
     <row r="98" spans="1:7">
       <c r="A98" s="44"/>
@@ -26605,8 +26596,8 @@
       <c r="E98" s="44" t="s">
         <v>1380</v>
       </c>
-      <c r="F98" s="116"/>
-      <c r="G98" s="116"/>
+      <c r="F98" s="117"/>
+      <c r="G98" s="117"/>
     </row>
     <row r="99" spans="1:7">
       <c r="A99" s="44"/>
@@ -26618,8 +26609,8 @@
       </c>
       <c r="D99" s="44"/>
       <c r="E99" s="44"/>
-      <c r="F99" s="116"/>
-      <c r="G99" s="116"/>
+      <c r="F99" s="117"/>
+      <c r="G99" s="117"/>
     </row>
     <row r="100" spans="1:7">
       <c r="A100" s="44"/>
@@ -26631,8 +26622,8 @@
       <c r="E100" s="44" t="s">
         <v>1384</v>
       </c>
-      <c r="F100" s="116"/>
-      <c r="G100" s="116"/>
+      <c r="F100" s="117"/>
+      <c r="G100" s="117"/>
     </row>
     <row r="101" spans="1:7">
       <c r="A101" s="44"/>
@@ -26644,8 +26635,8 @@
       <c r="E101" s="44" t="s">
         <v>1386</v>
       </c>
-      <c r="F101" s="116"/>
-      <c r="G101" s="116"/>
+      <c r="F101" s="117"/>
+      <c r="G101" s="117"/>
     </row>
     <row r="102" spans="1:7">
       <c r="A102" s="44"/>
@@ -26657,8 +26648,8 @@
       </c>
       <c r="D102" s="44"/>
       <c r="E102" s="44"/>
-      <c r="F102" s="116"/>
-      <c r="G102" s="116"/>
+      <c r="F102" s="117"/>
+      <c r="G102" s="117"/>
     </row>
     <row r="103" spans="1:7">
       <c r="A103" s="44"/>
@@ -26670,8 +26661,8 @@
       </c>
       <c r="D103" s="44"/>
       <c r="E103" s="44"/>
-      <c r="F103" s="116"/>
-      <c r="G103" s="116"/>
+      <c r="F103" s="117"/>
+      <c r="G103" s="117"/>
     </row>
     <row r="104" spans="1:7">
       <c r="A104" s="44"/>
@@ -26683,8 +26674,8 @@
       <c r="E104" s="44" t="s">
         <v>1392</v>
       </c>
-      <c r="F104" s="116"/>
-      <c r="G104" s="116"/>
+      <c r="F104" s="117"/>
+      <c r="G104" s="117"/>
     </row>
     <row r="105" spans="1:7">
       <c r="A105" s="44"/>
@@ -26696,8 +26687,8 @@
       <c r="E105" s="44" t="s">
         <v>1394</v>
       </c>
-      <c r="F105" s="116"/>
-      <c r="G105" s="116"/>
+      <c r="F105" s="117"/>
+      <c r="G105" s="117"/>
     </row>
     <row r="106" spans="1:7">
       <c r="A106" s="44"/>
@@ -26709,8 +26700,8 @@
       <c r="E106" s="44" t="s">
         <v>1199</v>
       </c>
-      <c r="F106" s="116"/>
-      <c r="G106" s="116"/>
+      <c r="F106" s="117"/>
+      <c r="G106" s="117"/>
     </row>
     <row r="107" spans="1:7">
       <c r="A107" s="44"/>
@@ -26722,8 +26713,8 @@
       <c r="E107" s="44" t="s">
         <v>1279</v>
       </c>
-      <c r="F107" s="116"/>
-      <c r="G107" s="116"/>
+      <c r="F107" s="117"/>
+      <c r="G107" s="117"/>
     </row>
     <row r="108" spans="1:7">
       <c r="A108" s="44"/>
@@ -26735,8 +26726,8 @@
       </c>
       <c r="D108" s="44"/>
       <c r="E108" s="44"/>
-      <c r="F108" s="116"/>
-      <c r="G108" s="116"/>
+      <c r="F108" s="117"/>
+      <c r="G108" s="117"/>
     </row>
     <row r="109" spans="1:7">
       <c r="A109" s="44"/>
@@ -26748,8 +26739,8 @@
       </c>
       <c r="D109" s="44"/>
       <c r="E109" s="44"/>
-      <c r="F109" s="116"/>
-      <c r="G109" s="116"/>
+      <c r="F109" s="117"/>
+      <c r="G109" s="117"/>
     </row>
     <row r="110" spans="1:7">
       <c r="A110" s="44"/>
@@ -26761,8 +26752,8 @@
       </c>
       <c r="D110" s="44"/>
       <c r="E110" s="44"/>
-      <c r="F110" s="116"/>
-      <c r="G110" s="116"/>
+      <c r="F110" s="117"/>
+      <c r="G110" s="117"/>
     </row>
     <row r="111" spans="1:7">
       <c r="A111" s="44"/>
@@ -26774,8 +26765,8 @@
       </c>
       <c r="D111" s="44"/>
       <c r="E111" s="44"/>
-      <c r="F111" s="116"/>
-      <c r="G111" s="116"/>
+      <c r="F111" s="117"/>
+      <c r="G111" s="117"/>
     </row>
     <row r="112" spans="1:7">
       <c r="A112" s="44"/>
@@ -26787,8 +26778,8 @@
       </c>
       <c r="D112" s="44"/>
       <c r="E112" s="44"/>
-      <c r="F112" s="116"/>
-      <c r="G112" s="116"/>
+      <c r="F112" s="117"/>
+      <c r="G112" s="117"/>
     </row>
     <row r="113" spans="1:7">
       <c r="A113" s="43" t="s">
@@ -26875,10 +26866,10 @@
       <c r="E118" s="44" t="s">
         <v>1419</v>
       </c>
-      <c r="F118" s="116" t="s">
+      <c r="F118" s="117" t="s">
         <v>1420</v>
       </c>
-      <c r="G118" s="116"/>
+      <c r="G118" s="117"/>
     </row>
     <row r="119" spans="1:7">
       <c r="A119" s="44"/>
@@ -26894,8 +26885,8 @@
       <c r="E119" s="44" t="s">
         <v>1424</v>
       </c>
-      <c r="F119" s="116"/>
-      <c r="G119" s="116"/>
+      <c r="F119" s="117"/>
+      <c r="G119" s="117"/>
     </row>
     <row r="120" spans="1:7">
       <c r="A120" t="s">
@@ -28380,10 +28371,10 @@
       </c>
       <c r="D279" s="44"/>
       <c r="E279" s="44"/>
-      <c r="F279" s="116" t="s">
+      <c r="F279" s="117" t="s">
         <v>1687</v>
       </c>
-      <c r="G279" s="116"/>
+      <c r="G279" s="117"/>
     </row>
     <row r="280" spans="1:7">
       <c r="A280" s="44"/>
@@ -28395,8 +28386,8 @@
       <c r="E280" s="44" t="s">
         <v>1689</v>
       </c>
-      <c r="F280" s="116"/>
-      <c r="G280" s="116"/>
+      <c r="F280" s="117"/>
+      <c r="G280" s="117"/>
     </row>
     <row r="281" spans="1:7">
       <c r="A281" s="44"/>
@@ -28408,8 +28399,8 @@
       </c>
       <c r="D281" s="44"/>
       <c r="E281" s="44"/>
-      <c r="F281" s="116"/>
-      <c r="G281" s="116"/>
+      <c r="F281" s="117"/>
+      <c r="G281" s="117"/>
     </row>
     <row r="282" spans="1:7">
       <c r="A282" s="44"/>
@@ -28425,8 +28416,8 @@
       <c r="E282" s="44" t="s">
         <v>1695</v>
       </c>
-      <c r="F282" s="116"/>
-      <c r="G282" s="116"/>
+      <c r="F282" s="117"/>
+      <c r="G282" s="117"/>
     </row>
     <row r="283" spans="1:7">
       <c r="A283" s="44"/>
@@ -28438,8 +28429,8 @@
       </c>
       <c r="D283" s="44"/>
       <c r="E283" s="44"/>
-      <c r="F283" s="116"/>
-      <c r="G283" s="116"/>
+      <c r="F283" s="117"/>
+      <c r="G283" s="117"/>
     </row>
     <row r="284" spans="1:7">
       <c r="A284" s="44"/>
@@ -28455,8 +28446,8 @@
       <c r="E284" s="44" t="s">
         <v>1701</v>
       </c>
-      <c r="F284" s="116"/>
-      <c r="G284" s="116"/>
+      <c r="F284" s="117"/>
+      <c r="G284" s="117"/>
     </row>
     <row r="285" spans="1:7">
       <c r="A285" s="44"/>
@@ -28468,8 +28459,8 @@
       <c r="E285" s="44" t="s">
         <v>1567</v>
       </c>
-      <c r="F285" s="116"/>
-      <c r="G285" s="116"/>
+      <c r="F285" s="117"/>
+      <c r="G285" s="117"/>
     </row>
     <row r="286" spans="1:7">
       <c r="A286" s="44"/>
@@ -28481,8 +28472,8 @@
       <c r="E286" s="44" t="s">
         <v>1203</v>
       </c>
-      <c r="F286" s="116"/>
-      <c r="G286" s="116"/>
+      <c r="F286" s="117"/>
+      <c r="G286" s="117"/>
     </row>
     <row r="287" spans="1:7">
       <c r="A287" s="44"/>
@@ -28494,8 +28485,8 @@
       <c r="E287" s="44" t="s">
         <v>1265</v>
       </c>
-      <c r="F287" s="116"/>
-      <c r="G287" s="116"/>
+      <c r="F287" s="117"/>
+      <c r="G287" s="117"/>
     </row>
     <row r="288" spans="1:7">
       <c r="A288" s="44"/>
@@ -28507,8 +28498,8 @@
       <c r="E288" s="44" t="s">
         <v>1281</v>
       </c>
-      <c r="F288" s="116"/>
-      <c r="G288" s="116"/>
+      <c r="F288" s="117"/>
+      <c r="G288" s="117"/>
     </row>
     <row r="289" spans="1:7">
       <c r="A289" s="44"/>
@@ -28520,8 +28511,8 @@
       <c r="E289" s="44" t="s">
         <v>1342</v>
       </c>
-      <c r="F289" s="116"/>
-      <c r="G289" s="116"/>
+      <c r="F289" s="117"/>
+      <c r="G289" s="117"/>
     </row>
     <row r="290" spans="1:7">
       <c r="A290" s="44"/>
@@ -28533,8 +28524,8 @@
       </c>
       <c r="D290" s="44"/>
       <c r="E290" s="44"/>
-      <c r="F290" s="116"/>
-      <c r="G290" s="116"/>
+      <c r="F290" s="117"/>
+      <c r="G290" s="117"/>
     </row>
     <row r="291" spans="1:7">
       <c r="A291" s="44"/>
@@ -28546,8 +28537,8 @@
       <c r="E291" s="44" t="s">
         <v>1705</v>
       </c>
-      <c r="F291" s="116"/>
-      <c r="G291" s="116"/>
+      <c r="F291" s="117"/>
+      <c r="G291" s="117"/>
     </row>
     <row r="292" spans="1:7">
       <c r="A292" s="44"/>
@@ -28559,8 +28550,8 @@
       <c r="E292" s="44" t="s">
         <v>1201</v>
       </c>
-      <c r="F292" s="116"/>
-      <c r="G292" s="116"/>
+      <c r="F292" s="117"/>
+      <c r="G292" s="117"/>
     </row>
     <row r="293" spans="1:7">
       <c r="A293" s="44"/>
@@ -28572,8 +28563,8 @@
       <c r="E293" s="44" t="s">
         <v>1571</v>
       </c>
-      <c r="F293" s="116"/>
-      <c r="G293" s="116"/>
+      <c r="F293" s="117"/>
+      <c r="G293" s="117"/>
     </row>
     <row r="294" spans="1:7">
       <c r="A294" s="44"/>
@@ -28585,8 +28576,8 @@
       <c r="E294" s="44" t="s">
         <v>1326</v>
       </c>
-      <c r="F294" s="116"/>
-      <c r="G294" s="116"/>
+      <c r="F294" s="117"/>
+      <c r="G294" s="117"/>
     </row>
     <row r="295" spans="1:7">
       <c r="A295" s="44"/>
@@ -28598,8 +28589,8 @@
       </c>
       <c r="D295" s="44"/>
       <c r="E295" s="44"/>
-      <c r="F295" s="116"/>
-      <c r="G295" s="116"/>
+      <c r="F295" s="117"/>
+      <c r="G295" s="117"/>
     </row>
     <row r="296" spans="1:7">
       <c r="A296" s="43" t="s">
@@ -28701,10 +28692,10 @@
       </c>
       <c r="D302" s="44"/>
       <c r="E302" s="44"/>
-      <c r="F302" s="116" t="s">
+      <c r="F302" s="117" t="s">
         <v>1711</v>
       </c>
-      <c r="G302" s="116" t="s">
+      <c r="G302" s="117" t="s">
         <v>1712</v>
       </c>
     </row>
@@ -28718,8 +28709,8 @@
       <c r="E303" s="44" t="s">
         <v>1689</v>
       </c>
-      <c r="F303" s="116"/>
-      <c r="G303" s="116"/>
+      <c r="F303" s="117"/>
+      <c r="G303" s="117"/>
     </row>
     <row r="304" spans="1:7">
       <c r="A304" s="43" t="s">
@@ -28925,10 +28916,10 @@
       </c>
       <c r="D316" s="44"/>
       <c r="E316" s="44"/>
-      <c r="F316" s="116" t="s">
+      <c r="F316" s="117" t="s">
         <v>1729</v>
       </c>
-      <c r="G316" s="116"/>
+      <c r="G316" s="117"/>
     </row>
     <row r="317" spans="1:7">
       <c r="A317" s="44"/>
@@ -28940,8 +28931,8 @@
       </c>
       <c r="D317" s="44"/>
       <c r="E317" s="44"/>
-      <c r="F317" s="116"/>
-      <c r="G317" s="116"/>
+      <c r="F317" s="117"/>
+      <c r="G317" s="117"/>
     </row>
     <row r="318" spans="1:7">
       <c r="A318" s="44"/>
@@ -28953,8 +28944,8 @@
       </c>
       <c r="D318" s="44"/>
       <c r="E318" s="44"/>
-      <c r="F318" s="116"/>
-      <c r="G318" s="116"/>
+      <c r="F318" s="117"/>
+      <c r="G318" s="117"/>
     </row>
     <row r="319" spans="1:7">
       <c r="A319" t="s">
@@ -30175,10 +30166,10 @@
       <c r="E450" s="44" t="s">
         <v>1981</v>
       </c>
-      <c r="F450" s="117" t="s">
+      <c r="F450" s="123" t="s">
         <v>1982</v>
       </c>
-      <c r="G450" s="116"/>
+      <c r="G450" s="117"/>
     </row>
     <row r="451" spans="1:7">
       <c r="A451" s="44"/>
@@ -30190,8 +30181,8 @@
       </c>
       <c r="D451" s="44"/>
       <c r="E451" s="44"/>
-      <c r="F451" s="117"/>
-      <c r="G451" s="116"/>
+      <c r="F451" s="123"/>
+      <c r="G451" s="117"/>
     </row>
     <row r="452" spans="1:7">
       <c r="A452" s="44"/>
@@ -30207,8 +30198,8 @@
       <c r="E452" s="44" t="s">
         <v>1988</v>
       </c>
-      <c r="F452" s="117"/>
-      <c r="G452" s="116"/>
+      <c r="F452" s="123"/>
+      <c r="G452" s="117"/>
     </row>
     <row r="453" spans="1:7">
       <c r="A453" s="44"/>
@@ -30220,8 +30211,8 @@
       <c r="E453" s="44" t="s">
         <v>1990</v>
       </c>
-      <c r="F453" s="117"/>
-      <c r="G453" s="116"/>
+      <c r="F453" s="123"/>
+      <c r="G453" s="117"/>
     </row>
     <row r="454" spans="1:7">
       <c r="A454" s="44"/>
@@ -30233,8 +30224,8 @@
       <c r="E454" s="44" t="s">
         <v>1992</v>
       </c>
-      <c r="F454" s="117"/>
-      <c r="G454" s="116"/>
+      <c r="F454" s="123"/>
+      <c r="G454" s="117"/>
     </row>
     <row r="455" spans="1:7">
       <c r="A455" s="44"/>
@@ -30246,8 +30237,8 @@
       </c>
       <c r="D455" s="44"/>
       <c r="E455" s="44"/>
-      <c r="F455" s="117"/>
-      <c r="G455" s="116"/>
+      <c r="F455" s="123"/>
+      <c r="G455" s="117"/>
     </row>
     <row r="456" spans="1:7">
       <c r="A456" s="44"/>
@@ -30259,8 +30250,8 @@
       </c>
       <c r="D456" s="44"/>
       <c r="E456" s="44"/>
-      <c r="F456" s="117"/>
-      <c r="G456" s="116"/>
+      <c r="F456" s="123"/>
+      <c r="G456" s="117"/>
     </row>
     <row r="457" spans="1:7">
       <c r="A457" s="44"/>
@@ -30272,8 +30263,8 @@
       </c>
       <c r="D457" s="44"/>
       <c r="E457" s="44"/>
-      <c r="F457" s="117"/>
-      <c r="G457" s="116"/>
+      <c r="F457" s="123"/>
+      <c r="G457" s="117"/>
     </row>
     <row r="458" spans="1:7">
       <c r="A458" s="44"/>
@@ -30285,8 +30276,8 @@
       </c>
       <c r="D458" s="44"/>
       <c r="E458" s="44"/>
-      <c r="F458" s="117"/>
-      <c r="G458" s="116"/>
+      <c r="F458" s="123"/>
+      <c r="G458" s="117"/>
     </row>
     <row r="459" spans="1:7">
       <c r="A459" s="44"/>
@@ -30298,8 +30289,8 @@
       </c>
       <c r="D459" s="44"/>
       <c r="E459" s="44"/>
-      <c r="F459" s="117"/>
-      <c r="G459" s="116"/>
+      <c r="F459" s="123"/>
+      <c r="G459" s="117"/>
     </row>
     <row r="460" spans="1:7">
       <c r="A460" s="44"/>
@@ -30311,8 +30302,8 @@
       </c>
       <c r="D460" s="44"/>
       <c r="E460" s="44"/>
-      <c r="F460" s="117"/>
-      <c r="G460" s="116"/>
+      <c r="F460" s="123"/>
+      <c r="G460" s="117"/>
     </row>
     <row r="461" spans="1:7">
       <c r="A461" s="44"/>
@@ -30324,8 +30315,8 @@
       <c r="E461" s="44" t="s">
         <v>2006</v>
       </c>
-      <c r="F461" s="117"/>
-      <c r="G461" s="116"/>
+      <c r="F461" s="123"/>
+      <c r="G461" s="117"/>
     </row>
     <row r="462" spans="1:7">
       <c r="A462" s="44"/>
@@ -30337,8 +30328,8 @@
       <c r="E462" s="44" t="s">
         <v>2008</v>
       </c>
-      <c r="F462" s="117"/>
-      <c r="G462" s="116"/>
+      <c r="F462" s="123"/>
+      <c r="G462" s="117"/>
     </row>
     <row r="463" spans="1:7">
       <c r="A463" s="44"/>
@@ -30354,8 +30345,8 @@
       <c r="E463" s="44" t="s">
         <v>2012</v>
       </c>
-      <c r="F463" s="117"/>
-      <c r="G463" s="116"/>
+      <c r="F463" s="123"/>
+      <c r="G463" s="117"/>
     </row>
     <row r="464" spans="1:7">
       <c r="A464" s="44"/>
@@ -30367,8 +30358,8 @@
       <c r="E464" s="44" t="s">
         <v>2014</v>
       </c>
-      <c r="F464" s="117"/>
-      <c r="G464" s="116"/>
+      <c r="F464" s="123"/>
+      <c r="G464" s="117"/>
     </row>
     <row r="465" spans="1:7">
       <c r="A465" s="44"/>
@@ -30380,8 +30371,8 @@
       </c>
       <c r="D465" s="44"/>
       <c r="E465" s="44"/>
-      <c r="F465" s="117"/>
-      <c r="G465" s="116"/>
+      <c r="F465" s="123"/>
+      <c r="G465" s="117"/>
     </row>
     <row r="466" spans="1:7">
       <c r="A466" s="44"/>
@@ -30393,8 +30384,8 @@
       </c>
       <c r="D466" s="44"/>
       <c r="E466" s="44"/>
-      <c r="F466" s="117"/>
-      <c r="G466" s="116"/>
+      <c r="F466" s="123"/>
+      <c r="G466" s="117"/>
     </row>
     <row r="467" spans="1:7">
       <c r="A467" s="44"/>
@@ -30406,8 +30397,8 @@
       </c>
       <c r="D467" s="44"/>
       <c r="E467" s="44"/>
-      <c r="F467" s="117"/>
-      <c r="G467" s="116"/>
+      <c r="F467" s="123"/>
+      <c r="G467" s="117"/>
     </row>
     <row r="468" spans="1:7">
       <c r="A468" s="44"/>
@@ -30419,8 +30410,8 @@
       </c>
       <c r="D468" s="44"/>
       <c r="E468" s="44"/>
-      <c r="F468" s="117"/>
-      <c r="G468" s="116"/>
+      <c r="F468" s="123"/>
+      <c r="G468" s="117"/>
     </row>
     <row r="469" spans="1:7">
       <c r="A469" s="44"/>
@@ -30432,8 +30423,8 @@
       </c>
       <c r="D469" s="44"/>
       <c r="E469" s="44"/>
-      <c r="F469" s="117"/>
-      <c r="G469" s="116"/>
+      <c r="F469" s="123"/>
+      <c r="G469" s="117"/>
     </row>
     <row r="470" spans="1:7">
       <c r="A470" s="44"/>
@@ -30445,8 +30436,8 @@
       </c>
       <c r="D470" s="44"/>
       <c r="E470" s="44"/>
-      <c r="F470" s="117"/>
-      <c r="G470" s="116"/>
+      <c r="F470" s="123"/>
+      <c r="G470" s="117"/>
     </row>
     <row r="471" spans="1:7">
       <c r="A471" s="44"/>
@@ -30458,8 +30449,8 @@
       </c>
       <c r="D471" s="44"/>
       <c r="E471" s="44"/>
-      <c r="F471" s="117"/>
-      <c r="G471" s="116"/>
+      <c r="F471" s="123"/>
+      <c r="G471" s="117"/>
     </row>
     <row r="472" spans="1:7">
       <c r="A472" s="44"/>
@@ -30471,8 +30462,8 @@
       </c>
       <c r="D472" s="44"/>
       <c r="E472" s="44"/>
-      <c r="F472" s="117"/>
-      <c r="G472" s="116"/>
+      <c r="F472" s="123"/>
+      <c r="G472" s="117"/>
     </row>
     <row r="473" spans="1:7">
       <c r="A473" s="44"/>
@@ -30484,8 +30475,8 @@
       </c>
       <c r="D473" s="44"/>
       <c r="E473" s="44"/>
-      <c r="F473" s="117"/>
-      <c r="G473" s="116"/>
+      <c r="F473" s="123"/>
+      <c r="G473" s="117"/>
     </row>
     <row r="474" spans="1:7">
       <c r="A474" s="44"/>
@@ -30501,7 +30492,7 @@
       <c r="E474" s="44" t="s">
         <v>2036</v>
       </c>
-      <c r="F474" s="117"/>
+      <c r="F474" s="123"/>
       <c r="G474" s="44"/>
     </row>
     <row r="475" spans="1:7">
@@ -30514,7 +30505,7 @@
       <c r="E475" s="44" t="s">
         <v>2038</v>
       </c>
-      <c r="F475" s="117"/>
+      <c r="F475" s="123"/>
       <c r="G475" s="44"/>
     </row>
     <row r="476" spans="1:7">
@@ -30523,7 +30514,7 @@
       <c r="C476" s="44"/>
       <c r="D476" s="44"/>
       <c r="E476" s="44"/>
-      <c r="F476" s="117"/>
+      <c r="F476" s="123"/>
       <c r="G476" s="44"/>
     </row>
     <row r="477" spans="1:7">
@@ -30695,6 +30686,22 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="F316:F318"/>
+    <mergeCell ref="G316:G318"/>
+    <mergeCell ref="F450:F476"/>
+    <mergeCell ref="G450:G473"/>
+    <mergeCell ref="F118:F119"/>
+    <mergeCell ref="G118:G119"/>
+    <mergeCell ref="F137:F139"/>
+    <mergeCell ref="G137:G139"/>
+    <mergeCell ref="F279:F295"/>
+    <mergeCell ref="G279:G295"/>
+    <mergeCell ref="F2:F6"/>
+    <mergeCell ref="G2:G6"/>
+    <mergeCell ref="F7:F13"/>
+    <mergeCell ref="G7:G13"/>
+    <mergeCell ref="F14:F18"/>
+    <mergeCell ref="G14:G18"/>
     <mergeCell ref="F19:F23"/>
     <mergeCell ref="G19:G23"/>
     <mergeCell ref="F304:F308"/>
@@ -30711,22 +30718,6 @@
     <mergeCell ref="G25:G31"/>
     <mergeCell ref="F64:F88"/>
     <mergeCell ref="G64:G88"/>
-    <mergeCell ref="F2:F6"/>
-    <mergeCell ref="G2:G6"/>
-    <mergeCell ref="F7:F13"/>
-    <mergeCell ref="G7:G13"/>
-    <mergeCell ref="F14:F18"/>
-    <mergeCell ref="G14:G18"/>
-    <mergeCell ref="F316:F318"/>
-    <mergeCell ref="G316:G318"/>
-    <mergeCell ref="F450:F476"/>
-    <mergeCell ref="G450:G473"/>
-    <mergeCell ref="F118:F119"/>
-    <mergeCell ref="G118:G119"/>
-    <mergeCell ref="F137:F139"/>
-    <mergeCell ref="G137:G139"/>
-    <mergeCell ref="F279:F295"/>
-    <mergeCell ref="G279:G295"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -31640,7 +31631,7 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
   </sheetData>
@@ -31652,6 +31643,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f" xsi:nil="true"/>
@@ -31668,16 +31668,57 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101005577104A61253744860FCC66480BADA8" ma:contentTypeVersion="18" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="63711f83cae101cfa77de3399d52e025">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="15b42a90-06dd-4669-ae82-892e5974bb2f" xmlns:ns3="c5dd6777-c59f-429e-841b-72020fd1fff4" xmlns:ns4="2d89f73c-94c0-4155-aa8d-969ee56d6579" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9da244f911df83ec31b8aa7de0186590" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="15b42a90-06dd-4669-ae82-892e5974bb2f"/>
@@ -31964,57 +32005,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8286976C-A32F-42CE-838F-E628DE116440}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E91276BE-0791-4771-952D-C50ABE3E5339}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -32032,15 +32031,15 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8286976C-A32F-42CE-838F-E628DE116440}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA3F46AF-7DEC-42CD-98A3-4934B1C64918}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9CF615A7-8B4A-4E31-8F9E-482FE203A4DA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -32058,12 +32057,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA3F46AF-7DEC-42CD-98A3-4934B1C64918}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>